<commit_message>
Price tracker: update run data (2026-10-16)
</commit_message>
<xml_diff>
--- a/Home Wishlist.xlsx
+++ b/Home Wishlist.xlsx
@@ -23,9 +23,9 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="169" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -71,7 +71,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -80,8 +80,10 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2129,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK46"/>
+  <dimension ref="A1:AK55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5037,7 +5039,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -5071,10 +5073,10 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="9" t="n">
+      <c r="K25" s="11" t="n">
         <v>12.37</v>
       </c>
-      <c r="O25" s="9" t="n">
+      <c r="O25" s="11" t="n">
         <v>10.12</v>
       </c>
       <c r="P25" t="inlineStr">
@@ -5088,7 +5090,7 @@
       <c r="R25" t="n">
         <v>3</v>
       </c>
-      <c r="T25" s="9" t="n">
+      <c r="T25" s="11" t="n">
         <v>13.49</v>
       </c>
       <c r="U25" t="inlineStr">
@@ -5101,7 +5103,7 @@
           <t>thirdreality.com: [success] $13.49 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $40.49 in stock - Shopify .js; identity validated (page_metadata)</t>
         </is>
       </c>
-      <c r="W25" s="9" t="n">
+      <c r="W25" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="X25" t="inlineStr">
@@ -5109,16 +5111,16 @@
           <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
         </is>
       </c>
-      <c r="Y25" s="9" t="n">
+      <c r="Y25" s="11" t="n">
         <v>13.49</v>
       </c>
       <c r="Z25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA25" s="9" t="n">
+      <c r="AA25" s="11" t="n">
         <v>10.12</v>
       </c>
-      <c r="AB25" s="9" t="n">
+      <c r="AB25" s="11" t="n">
         <v>14.54</v>
       </c>
       <c r="AC25" t="n">
@@ -5129,7 +5131,7 @@
           <t>2 x single @ THIRDREALITY Store ($13.49) = $26.98 for 2 unit(s) ($13.49/unit)</t>
         </is>
       </c>
-      <c r="AE25" s="9" t="n">
+      <c r="AE25" s="11" t="n">
         <v>26.98</v>
       </c>
       <c r="AF25" t="inlineStr">
@@ -5164,7 +5166,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -5198,13 +5200,13 @@
       <c r="J26" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="9" t="n">
+      <c r="K26" s="11" t="n">
         <v>219</v>
       </c>
-      <c r="M26" s="9" t="n">
+      <c r="M26" s="11" t="n">
         <v>219</v>
       </c>
-      <c r="O26" s="9" t="n">
+      <c r="O26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="P26" t="inlineStr">
@@ -5218,7 +5220,7 @@
       <c r="R26" t="n">
         <v>1</v>
       </c>
-      <c r="T26" s="9" t="n">
+      <c r="T26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="U26" t="inlineStr">
@@ -5231,7 +5233,7 @@
           <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $1,016.00 via Google Shopping fallback (market_snapshot, not verified)</t>
         </is>
       </c>
-      <c r="W26" s="9" t="n">
+      <c r="W26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="X26" t="inlineStr">
@@ -5239,16 +5241,16 @@
           <t>msrp_regular: manufacturer price at Sonos Direct</t>
         </is>
       </c>
-      <c r="Y26" s="9" t="n">
+      <c r="Y26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="Z26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA26" s="9" t="n">
+      <c r="AA26" s="11" t="n">
         <v>219</v>
       </c>
-      <c r="AB26" s="9" t="n">
+      <c r="AB26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="AC26" t="n">
@@ -5259,7 +5261,7 @@
           <t>1 x single @ Sonos Direct ($219.00) = $219.00 for 1 unit(s) ($219.00/unit)</t>
         </is>
       </c>
-      <c r="AE26" s="9" t="n">
+      <c r="AE26" s="11" t="n">
         <v>219</v>
       </c>
       <c r="AF26" t="inlineStr">
@@ -5294,7 +5296,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -5328,13 +5330,13 @@
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="9" t="n">
+      <c r="K27" s="11" t="n">
         <v>1098.39</v>
       </c>
-      <c r="M27" s="9" t="n">
+      <c r="M27" s="11" t="n">
         <v>1097.99</v>
       </c>
-      <c r="O27" s="9" t="n">
+      <c r="O27" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="P27" t="inlineStr">
@@ -5348,7 +5350,7 @@
       <c r="R27" t="n">
         <v>5</v>
       </c>
-      <c r="T27" s="9" t="n">
+      <c r="T27" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="U27" t="inlineStr">
@@ -5361,7 +5363,7 @@
           <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $2,101.00 via Google Shopping fallback (market_snapshot, not verified) | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (browser render); identity validated (product_url)</t>
         </is>
       </c>
-      <c r="W27" s="9" t="n">
+      <c r="W27" s="11" t="n">
         <v>1499.99</v>
       </c>
       <c r="X27" t="inlineStr">
@@ -5369,16 +5371,16 @@
           <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
         </is>
       </c>
-      <c r="Y27" s="9" t="n">
+      <c r="Y27" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="Z27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA27" s="9" t="n">
+      <c r="AA27" s="11" t="n">
         <v>1097.99</v>
       </c>
-      <c r="AB27" s="9" t="n">
+      <c r="AB27" s="11" t="n">
         <v>1098.41</v>
       </c>
       <c r="AC27" t="n">
@@ -5389,7 +5391,7 @@
           <t>1 x single @ Amazon ($1,097.99) = $1,097.99 for 1 unit(s) ($1,097.99/unit)</t>
         </is>
       </c>
-      <c r="AE27" s="9" t="n">
+      <c r="AE27" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="AF27" t="inlineStr">
@@ -5424,7 +5426,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -5458,13 +5460,13 @@
       <c r="J28" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="9" t="n">
+      <c r="K28" s="11" t="n">
         <v>319.99</v>
       </c>
-      <c r="M28" s="9" t="n">
+      <c r="M28" s="11" t="n">
         <v>319.99</v>
       </c>
-      <c r="O28" s="9" t="n">
+      <c r="O28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="P28" t="inlineStr">
@@ -5478,7 +5480,7 @@
       <c r="R28" t="n">
         <v>2</v>
       </c>
-      <c r="T28" s="9" t="n">
+      <c r="T28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="U28" t="inlineStr">
@@ -5491,7 +5493,7 @@
           <t>amazon.com: [success] $319.99 stock unknown - visible price markup (browser render); identity validated (product_url) | philips-hue.com: [unavailable] $319.99 OUT OF STOCK - JSON-LD; identity validated (gtin)</t>
         </is>
       </c>
-      <c r="W28" s="9" t="n">
+      <c r="W28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="X28" t="inlineStr">
@@ -5499,16 +5501,16 @@
           <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
         </is>
       </c>
-      <c r="Y28" s="9" t="n">
+      <c r="Y28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="Z28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA28" s="9" t="n">
+      <c r="AA28" s="11" t="n">
         <v>239.97</v>
       </c>
-      <c r="AB28" s="9" t="n">
+      <c r="AB28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="AC28" t="n">
@@ -5519,7 +5521,7 @@
           <t>1 x single @ Amazon ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
         </is>
       </c>
-      <c r="AE28" s="9" t="n">
+      <c r="AE28" s="11" t="n">
         <v>319.99</v>
       </c>
       <c r="AF28" t="inlineStr">
@@ -5554,7 +5556,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n">
+      <c r="A29" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -5588,13 +5590,13 @@
       <c r="J29" t="n">
         <v>0</v>
       </c>
-      <c r="K29" s="9" t="n">
+      <c r="K29" s="11" t="n">
         <v>146.66</v>
       </c>
-      <c r="M29" s="9" t="n">
+      <c r="M29" s="11" t="n">
         <v>169.99</v>
       </c>
-      <c r="O29" s="9" t="n">
+      <c r="O29" s="11" t="n">
         <v>169.99</v>
       </c>
       <c r="P29" t="inlineStr">
@@ -5608,7 +5610,7 @@
       <c r="R29" t="n">
         <v>3</v>
       </c>
-      <c r="T29" s="9" t="n">
+      <c r="T29" s="11" t="n">
         <v>169.99</v>
       </c>
       <c r="U29" t="inlineStr">
@@ -5621,7 +5623,7 @@
           <t>amazon.com: [success] $169.99 stock unknown - visible price markup (browser render); identity validated (product_url) | us.govee.com: [success] $169.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
         </is>
       </c>
-      <c r="W29" s="9" t="n">
+      <c r="W29" s="11" t="n">
         <v>169.99</v>
       </c>
       <c r="X29" t="inlineStr">
@@ -5629,16 +5631,16 @@
           <t>msrp_regular: manufacturer price at Govee</t>
         </is>
       </c>
-      <c r="Y29" s="9" t="n">
+      <c r="Y29" s="11" t="n">
         <v>169.99</v>
       </c>
       <c r="Z29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA29" s="9" t="n">
+      <c r="AA29" s="11" t="n">
         <v>74.98999999999999</v>
       </c>
-      <c r="AB29" s="9" t="n">
+      <c r="AB29" s="11" t="n">
         <v>162.64</v>
       </c>
       <c r="AC29" t="n">
@@ -5649,7 +5651,7 @@
           <t>2 x single @ Govee ($169.99) = $339.98 for 2 unit(s) ($169.99/unit)</t>
         </is>
       </c>
-      <c r="AE29" s="9" t="n">
+      <c r="AE29" s="11" t="n">
         <v>339.98</v>
       </c>
       <c r="AF29" t="inlineStr">
@@ -5684,7 +5686,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="n">
+      <c r="A30" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -5718,10 +5720,10 @@
       <c r="J30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" s="9" t="n">
+      <c r="L30" s="11" t="n">
         <v>191.49</v>
       </c>
-      <c r="O30" s="9" t="n">
+      <c r="O30" s="11" t="n">
         <v>191.49</v>
       </c>
       <c r="P30" t="inlineStr">
@@ -5758,7 +5760,7 @@
           <t>1 x single @ reebelo.com ($191.49, refurbished) = $191.49 for 1 unit(s) ($191.49/unit)</t>
         </is>
       </c>
-      <c r="AE30" s="9" t="n">
+      <c r="AE30" s="11" t="n">
         <v>191.49</v>
       </c>
       <c r="AF30" t="inlineStr">
@@ -5793,7 +5795,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="n">
+      <c r="A31" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -5890,7 +5892,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="n">
+      <c r="A32" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -5987,7 +5989,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="n">
+      <c r="A33" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -6084,7 +6086,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -6181,7 +6183,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="n">
+      <c r="A35" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -6215,10 +6217,10 @@
       <c r="J35" t="n">
         <v>0</v>
       </c>
-      <c r="K35" s="9" t="n">
+      <c r="K35" s="11" t="n">
         <v>249.99</v>
       </c>
-      <c r="O35" s="9" t="n">
+      <c r="O35" s="11" t="n">
         <v>249.99</v>
       </c>
       <c r="P35" t="inlineStr">
@@ -6232,7 +6234,7 @@
       <c r="R35" t="n">
         <v>1</v>
       </c>
-      <c r="T35" s="9" t="n">
+      <c r="T35" s="11" t="n">
         <v>249.99</v>
       </c>
       <c r="U35" t="inlineStr">
@@ -6245,7 +6247,7 @@
           <t>amazon.com: [success] $249.99 stock unknown - visible price markup (browser render); redirected to https://www.amazon.com/WallBeyond-Mounted-Bedroom-Leaning-Hanging/dp/B0GSFK8V4L/; identity validated (title)</t>
         </is>
       </c>
-      <c r="W35" s="9" t="n">
+      <c r="W35" s="11" t="n">
         <v>249.99</v>
       </c>
       <c r="X35" t="inlineStr">
@@ -6253,7 +6255,7 @@
           <t>verified_current: verified current price (no regular price published)</t>
         </is>
       </c>
-      <c r="AA35" s="9" t="n">
+      <c r="AA35" s="11" t="n">
         <v>249.99</v>
       </c>
       <c r="AC35" t="n">
@@ -6264,7 +6266,7 @@
           <t>1 x single @ Amazon ($249.99) = $249.99 for 1 unit(s) ($249.99/unit)</t>
         </is>
       </c>
-      <c r="AE35" s="9" t="n">
+      <c r="AE35" s="11" t="n">
         <v>249.99</v>
       </c>
       <c r="AF35" t="inlineStr">
@@ -6299,7 +6301,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="n">
+      <c r="A36" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -6351,7 +6353,7 @@
           <t>etsy.com: [blocked] FAILED - circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)); browser: circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)) -&gt; $63.00 from Etsy - Seller via Google Shopping (market_snapshot, not verified)</t>
         </is>
       </c>
-      <c r="W36" s="9" t="n">
+      <c r="W36" s="11" t="n">
         <v>299.5</v>
       </c>
       <c r="X36" t="inlineStr">
@@ -6399,7 +6401,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n">
+      <c r="A37" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -6433,10 +6435,10 @@
       <c r="J37" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="9" t="n">
+      <c r="K37" s="11" t="n">
         <v>24.99</v>
       </c>
-      <c r="O37" s="9" t="n">
+      <c r="O37" s="11" t="n">
         <v>24.99</v>
       </c>
       <c r="P37" t="inlineStr">
@@ -6450,7 +6452,7 @@
       <c r="R37" t="n">
         <v>1</v>
       </c>
-      <c r="T37" s="9" t="n">
+      <c r="T37" s="11" t="n">
         <v>24.99</v>
       </c>
       <c r="U37" t="inlineStr">
@@ -6463,7 +6465,7 @@
           <t>amazon.com: [success] $24.99 stock unknown - visible price markup (browser render); identity validated (mpn)</t>
         </is>
       </c>
-      <c r="W37" s="9" t="n">
+      <c r="W37" s="11" t="n">
         <v>24.99</v>
       </c>
       <c r="X37" t="inlineStr">
@@ -6471,7 +6473,7 @@
           <t>verified_current: verified current price (no regular price published)</t>
         </is>
       </c>
-      <c r="AA37" s="9" t="n">
+      <c r="AA37" s="11" t="n">
         <v>24.99</v>
       </c>
       <c r="AC37" t="n">
@@ -6482,7 +6484,7 @@
           <t>3 x single @ Amazon ($24.99) = $74.97 for 3 unit(s) ($24.99/unit)</t>
         </is>
       </c>
-      <c r="AE37" s="9" t="n">
+      <c r="AE37" s="11" t="n">
         <v>74.97</v>
       </c>
       <c r="AF37" t="inlineStr">
@@ -6517,7 +6519,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="n">
+      <c r="A38" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -6551,10 +6553,10 @@
       <c r="J38" t="n">
         <v>1</v>
       </c>
-      <c r="K38" s="9" t="n">
+      <c r="K38" s="11" t="n">
         <v>17.66</v>
       </c>
-      <c r="O38" s="9" t="n">
+      <c r="O38" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="P38" t="inlineStr">
@@ -6568,7 +6570,7 @@
       <c r="R38" t="n">
         <v>3</v>
       </c>
-      <c r="T38" s="9" t="n">
+      <c r="T38" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="U38" t="inlineStr">
@@ -6581,7 +6583,7 @@
           <t>thirdreality.com: [success] $14.99 in stock - Shopify .js; identity validated (product_url) (+3 variants)</t>
         </is>
       </c>
-      <c r="W38" s="9" t="n">
+      <c r="W38" s="11" t="n">
         <v>19.99</v>
       </c>
       <c r="X38" t="inlineStr">
@@ -6589,7 +6591,7 @@
           <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
         </is>
       </c>
-      <c r="AA38" s="9" t="n">
+      <c r="AA38" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="AC38" t="n">
@@ -6600,7 +6602,7 @@
           <t>5 x single @ THIRDREALITY Store ($14.99) = $74.95 for 5 unit(s) ($14.99/unit)</t>
         </is>
       </c>
-      <c r="AE38" s="9" t="n">
+      <c r="AE38" s="11" t="n">
         <v>74.95</v>
       </c>
       <c r="AF38" t="inlineStr">
@@ -6635,7 +6637,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="n">
+      <c r="A39" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -6669,10 +6671,10 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
-      <c r="K39" s="9" t="n">
+      <c r="K39" s="11" t="n">
         <v>64</v>
       </c>
-      <c r="O39" s="9" t="n">
+      <c r="O39" s="11" t="n">
         <v>64</v>
       </c>
       <c r="P39" t="inlineStr">
@@ -6686,7 +6688,7 @@
       <c r="R39" t="n">
         <v>1</v>
       </c>
-      <c r="T39" s="9" t="n">
+      <c r="T39" s="11" t="n">
         <v>64</v>
       </c>
       <c r="U39" t="inlineStr">
@@ -6699,7 +6701,7 @@
           <t>everythingsmart.io: [success] $64.00 in stock - Shopify .js; identity validated (title)</t>
         </is>
       </c>
-      <c r="W39" s="9" t="n">
+      <c r="W39" s="11" t="n">
         <v>64</v>
       </c>
       <c r="X39" t="inlineStr">
@@ -6707,7 +6709,7 @@
           <t>msrp_regular: manufacturer price at everythingsmart.io</t>
         </is>
       </c>
-      <c r="AA39" s="9" t="n">
+      <c r="AA39" s="11" t="n">
         <v>64</v>
       </c>
       <c r="AC39" t="n">
@@ -6718,7 +6720,7 @@
           <t>2 x single @ everythingsmart.io ($64.00) = $128.00 for 2 unit(s) ($64.00/unit)</t>
         </is>
       </c>
-      <c r="AE39" s="9" t="n">
+      <c r="AE39" s="11" t="n">
         <v>128</v>
       </c>
       <c r="AF39" t="inlineStr">
@@ -6753,7 +6755,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="n">
+      <c r="A40" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -6850,7 +6852,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="n">
+      <c r="A41" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -6884,7 +6886,7 @@
       <c r="J41" t="n">
         <v>0</v>
       </c>
-      <c r="K41" s="9" t="n">
+      <c r="K41" s="11" t="n">
         <v>17.07</v>
       </c>
       <c r="P41" t="inlineStr">
@@ -6953,7 +6955,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="n">
+      <c r="A42" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -7050,7 +7052,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="n">
+      <c r="A43" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -7147,7 +7149,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="n">
+      <c r="A44" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -7244,7 +7246,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="n">
+      <c r="A45" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -7341,7 +7343,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="n">
+      <c r="A46" s="10" t="n">
         <v>46308.82774305555</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -7434,6 +7436,1116 @@
       <c r="AK46" t="inlineStr">
         <is>
           <t>Yes (run 2 in a row): Etsy - Seller (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>17</v>
+      </c>
+      <c r="F47" t="n">
+        <v>12</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="11" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="M47" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="O47" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 15 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>5</v>
+      </c>
+      <c r="R47" t="n">
+        <v>4</v>
+      </c>
+      <c r="T47" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $13.49 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $40.49 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W47" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y47" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="Z47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="AB47" s="11" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>2 x single @ THIRDREALITY Store ($13.49) = $26.98 for 2 unit(s) ($13.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE47" s="11" t="n">
+        <v>26.98</v>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1SPD1Z, P1SPD4Z | brand THIRDREALITY</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 3</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>success 3 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>12</v>
+      </c>
+      <c r="F48" t="n">
+        <v>7</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="M48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="O48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 11 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>1</v>
+      </c>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="T48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>verified: Sonos Direct (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $1,016.00 via Google Shopping fallback (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="W48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Sonos Direct</t>
+        </is>
+      </c>
+      <c r="Y48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="Z48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AB48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>1 x single @ Sonos Direct ($219.00) = $219.00 for 1 unit(s) ($219.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE48" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>GTIN 840136802846 | MPN/SKU RAYG1US1BLK | brand Sonos</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>Yes (run 4 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>5</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>27</v>
+      </c>
+      <c r="F49" t="n">
+        <v>13</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="11" t="n">
+        <v>1098.39</v>
+      </c>
+      <c r="M49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="O49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 25 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>5</v>
+      </c>
+      <c r="R49" t="n">
+        <v>5</v>
+      </c>
+      <c r="T49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (browser render); identity validated (product_url)</t>
+        </is>
+      </c>
+      <c r="W49" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
+        </is>
+      </c>
+      <c r="Y49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="Z49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AB49" s="11" t="n">
+        <v>1098.28</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>1 x single @ Amazon ($1,097.99) = $1,097.99 for 1 unit(s) ($1,097.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>GTIN 887276934532 | MPN/SKU QN50QN90FAFXZA | brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 3</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | unavailable 1 (samsung.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>Yes (run 4 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Philips Hue Twilight Lamp Black</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="M50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="O50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (2 verified merchant prices; last discovery 2.9d ago (&lt; 6d) - credit saved) | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>2</v>
+      </c>
+      <c r="R50" t="n">
+        <v>2</v>
+      </c>
+      <c r="T50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Philips Hue Direct (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $319.99 stock unknown - visible price markup (browser render); identity validated (product_url) | philips-hue.com: [success] $319.99 in stock - JSON-LD; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
+        </is>
+      </c>
+      <c r="Y50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="Z50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA50" s="11" t="n">
+        <v>239.97</v>
+      </c>
+      <c r="AB50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>1 x single @ Philips Hue Direct ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE50" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>GTIN 46677585631 | MPN/SKU 929003711501 | brand Philips Hue</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>success 2 | api_unavailable 1 (eBay) | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>Not run (SerpApi unavailable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>6</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="11" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="M51" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="O51" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (2 verified merchant prices; last discovery 2.9d ago (&lt; 6d) - credit saved)</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>3</v>
+      </c>
+      <c r="R51" t="n">
+        <v>3</v>
+      </c>
+      <c r="T51" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Govee (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $169.99 stock unknown - visible price markup (browser render); identity validated (product_url) | us.govee.com: [success] $169.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
+        </is>
+      </c>
+      <c r="W51" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Govee</t>
+        </is>
+      </c>
+      <c r="Y51" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="Z51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="11" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="AB51" s="11" t="n">
+        <v>164.84</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>2 x single @ Govee ($169.99) = $339.98 for 2 unit(s) ($169.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE51" s="11" t="n">
+        <v>339.98</v>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>GTIN 810172723184 | MPN/SKU H1AA5, H1AA2 | brand Govee</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>verified_direct 3</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>11</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy Tab A9 plus silver</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>40</v>
+      </c>
+      <c r="F52" t="n">
+        <v>22</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="11" t="n">
+        <v>191.49</v>
+      </c>
+      <c r="O52" s="11" t="n">
+        <v>191.49</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Samsung, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 4 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | Avg (Resale) from only 1 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>9</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1</v>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>ebay.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) | reebelo.com: [success] $158.48 in stock - JSON-LD; identity validated (product_url) (+3 variants)</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>1 x single @ reebelo.com ($191.49, refurbished) = $191.49 for 1 unit(s) ($191.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE52" s="11" t="n">
+        <v>191.49</v>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>verified_direct 4 | market_snapshot 5</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (ebay.com) | api_unavailable 1 (eBay) | skipped 5 (Dell, Home Depot, Microcenter, Samsung, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): ebay.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>8</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="O53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | 5 Google row(s) from vendors with a working Product URL ignored | SerpApi: success 1 listings</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>1</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1</v>
+      </c>
+      <c r="T53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>verified: merachfit.com (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>merachfit.com: [success] $299.99 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W53" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>msrp_regular: retailer regular/list price at merachfit.com</t>
+        </is>
+      </c>
+      <c r="Y53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="Z53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AB53" s="11" t="n">
+        <v>320.99</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>1 x single @ merachfit.com ($299.99) = $299.99 for 1 unit(s) ($299.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE53" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>MPN/SKU MR-T25B2-US | brand MERACH</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>9</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Costway 47x24 Treadmill May Large</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | wayfair.com: Product URL failed (identity_mismatch); same-vendor fallback timeout_network (request failed) | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>wayfair.com: [identity_mismatch] $31.90 stock unknown - page is not this product - Product URL page conflicts: accessory word 'protector'; IDENTITY MISMATCH (excluded) -&gt; same-vendor fallback: timeout_network (request failed)</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>brand Costway</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr">
+        <is>
+          <t>identity_mismatch 1 (wayfair.com) | timeout_network 2 (Google Shopping, wayfair.com (Google Shopping)) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): wayfair.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n">
+        <v>46311.72460648148</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Philips Hue Essential Smart LED A19 Bulb</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>40</v>
+      </c>
+      <c r="F55" t="n">
+        <v>24</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="O55" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Philips Hue Direct, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | verified price up 7.9% vs prior $4.06 (2026-10-10)</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>1</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1</v>
+      </c>
+      <c r="T55" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $17.50 stock unknown - visible price markup (browser render); identity validated (title)</t>
+        </is>
+      </c>
+      <c r="W55" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y55" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="Z55" s="5" t="n">
+        <v>0.0788</v>
+      </c>
+      <c r="AA55" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="AB55" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>2 x 4-pack @ Amazon ($17.50) = $35.00 for 8 unit(s) ($4.38/unit)</t>
+        </is>
+      </c>
+      <c r="AE55" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>MPN/SKU 592592 | brand Hue</t>
+        </is>
+      </c>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH55" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 5 (Dell, Home Depot, Microcenter, Philips Hue Direct, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI55" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK55" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -7449,7 +8561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF14"/>
+  <dimension ref="A1:AF20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -8612,10 +9724,10 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="H10" t="inlineStr">
@@ -8638,7 +9750,7 @@
           <t>new</t>
         </is>
       </c>
-      <c r="L10" s="9" t="n">
+      <c r="L10" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="M10" t="n">
@@ -8657,7 +9769,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8668,7 +9779,7 @@
           <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
         </is>
       </c>
-      <c r="T10" s="9" t="n">
+      <c r="T10" s="11" t="n">
         <v>1499.99</v>
       </c>
       <c r="U10" s="5" t="n">
@@ -8694,8 +9805,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -8734,10 +9843,10 @@
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="H11" t="inlineStr">
@@ -8760,7 +9869,7 @@
           <t>new</t>
         </is>
       </c>
-      <c r="L11" s="9" t="n">
+      <c r="L11" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="M11" t="n">
@@ -8779,7 +9888,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8790,7 +9898,7 @@
           <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a WireLogic Ruby 8ft Ultra High Speed 4K-8K-10K HDMI Cable</t>
         </is>
       </c>
-      <c r="T11" s="9" t="n">
+      <c r="T11" s="11" t="n">
         <v>1499.99</v>
       </c>
       <c r="U11" s="5" t="n">
@@ -8811,7 +9919,7 @@
           <t>msrp_regular</t>
         </is>
       </c>
-      <c r="Z11" s="9" t="n">
+      <c r="Z11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="AA11" t="inlineStr">
@@ -8819,8 +9927,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -8859,10 +9965,10 @@
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="H12" t="inlineStr">
@@ -8885,7 +9991,7 @@
           <t>new</t>
         </is>
       </c>
-      <c r="L12" s="9" t="n">
+      <c r="L12" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="M12" t="n">
@@ -8904,7 +10010,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -8915,7 +10020,7 @@
           <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV FIXED-Mount-43-90 TV Mount for 43"-98" TVs and Amber Protection 3</t>
         </is>
       </c>
-      <c r="T12" s="9" t="n">
+      <c r="T12" s="11" t="n">
         <v>1499.99</v>
       </c>
       <c r="U12" s="5" t="n">
@@ -8936,7 +10041,7 @@
           <t>msrp_regular</t>
         </is>
       </c>
-      <c r="Z12" s="9" t="n">
+      <c r="Z12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="AA12" t="inlineStr">
@@ -8944,8 +10049,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -8984,10 +10087,10 @@
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="11" t="n">
         <v>900</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="H13" t="inlineStr">
@@ -9010,7 +10113,7 @@
           <t>new</t>
         </is>
       </c>
-      <c r="L13" s="9" t="n">
+      <c r="L13" s="11" t="n">
         <v>1097.99</v>
       </c>
       <c r="M13" t="n">
@@ -9029,7 +10132,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -9040,7 +10142,7 @@
           <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
         </is>
       </c>
-      <c r="T13" s="9" t="n">
+      <c r="T13" s="11" t="n">
         <v>1499.99</v>
       </c>
       <c r="U13" s="5" t="n">
@@ -9061,7 +10163,7 @@
           <t>msrp_regular</t>
         </is>
       </c>
-      <c r="Z13" s="9" t="n">
+      <c r="Z13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="AA13" t="inlineStr">
@@ -9069,8 +10171,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -9109,10 +10209,10 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="H14" t="inlineStr">
@@ -9135,7 +10235,7 @@
           <t>new</t>
         </is>
       </c>
-      <c r="L14" s="9" t="n">
+      <c r="L14" s="11" t="n">
         <v>14.99</v>
       </c>
       <c r="M14" t="n">
@@ -9154,7 +10254,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -9165,7 +10264,7 @@
           <t>Motion Sensor - Single Pack</t>
         </is>
       </c>
-      <c r="T14" s="9" t="n">
+      <c r="T14" s="11" t="n">
         <v>19.99</v>
       </c>
       <c r="U14" s="5" t="n">
@@ -9186,7 +10285,7 @@
           <t>msrp_regular</t>
         </is>
       </c>
-      <c r="Y14" s="9" t="n">
+      <c r="Y14" s="11" t="n">
         <v>19.99</v>
       </c>
       <c r="AA14" t="inlineStr">
@@ -9194,8 +10293,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -9209,6 +10306,753 @@
       <c r="AF14" t="inlineStr">
         <is>
           <t>2026-10-13 19:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/smart-plug-gen3?variant=51228333867232</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>40.49</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0.3253</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>below 30d verified median $13.49 [new pool]</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Smart Plug Gen3 - 4-Pack</t>
+        </is>
+      </c>
+      <c r="T15" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="U15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>verified_pack</t>
+        </is>
+      </c>
+      <c r="Y15" s="11" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>7ae42c2156d2</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DXMVWFMC?plpRedirect=mhFallback&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
+        </is>
+      </c>
+      <c r="T16" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U16" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>64b642ed05e3</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:1015009314264515626,productid:14088425758659728466,headlineOfferDocid:1709814953679449319,imageDocid:7051938930816075256,gpcid:2064809066823823720,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a WireLogic Ruby 8ft Ultra High Speed 4K-8K-10K HDMI Cable</t>
+        </is>
+      </c>
+      <c r="T17" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U17" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-13</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>f3092c330421</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:16585649947930718367,productid:7930562881768223502,headlineOfferDocid:15992245985528261990,imageDocid:6687171378154213687,gpcid:1734279301782434442,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV FIXED-Mount-43-90 TV Mount for 43"-98" TVs and Amber Protection 3</t>
+        </is>
+      </c>
+      <c r="T18" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U18" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-13</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>9044cf35f8f1</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:9212013035633147240,productid:507093706451136505,headlineOfferDocid:15716683707371333184,imageDocid:13820267211841367837,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
+        </is>
+      </c>
+      <c r="T19" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U19" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>21297db3f4f0</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>gh-38939235833</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://merachfit.com/products/novawalk-w50-trekpad</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>merachfit.com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $479.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="T20" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="U20" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Y20" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>8fc2f05d8e66</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price tracker: update run data (2026-10-19)
</commit_message>
<xml_diff>
--- a/Home Wishlist.xlsx
+++ b/Home Wishlist.xlsx
@@ -2131,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK55"/>
+  <dimension ref="A1:AK75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8549,6 +8549,2261 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>16</v>
+      </c>
+      <c r="F56" t="n">
+        <v>12</v>
+      </c>
+      <c r="G56" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" t="n">
+        <v>2</v>
+      </c>
+      <c r="I56" t="n">
+        <v>1</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="11" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="M56" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="O56" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 14 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
+        <v>4</v>
+      </c>
+      <c r="R56" t="n">
+        <v>4</v>
+      </c>
+      <c r="T56" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $13.49 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $40.49 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W56" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y56" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="Z56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA56" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="AB56" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>2 x single @ THIRDREALITY Store ($13.49) = $26.98 for 2 unit(s) ($13.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE56" s="11" t="n">
+        <v>26.98</v>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1SPD1Z, P1SPD4Z | brand THIRDREALITY</t>
+        </is>
+      </c>
+      <c r="AG56" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 2</t>
+        </is>
+      </c>
+      <c r="AH56" t="inlineStr">
+        <is>
+          <t>success 3 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI56" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>19</v>
+      </c>
+      <c r="F57" t="n">
+        <v>14</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="n">
+        <v>2</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="11" t="n">
+        <v>233</v>
+      </c>
+      <c r="L57" s="11" t="n">
+        <v>165.99</v>
+      </c>
+      <c r="M57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="O57" s="11" t="n">
+        <v>141.99</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 17 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | Avg (Resale) from only 2 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
+        <v>5</v>
+      </c>
+      <c r="R57" t="n">
+        <v>3</v>
+      </c>
+      <c r="S57" t="n">
+        <v>2</v>
+      </c>
+      <c r="T57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>verified: Sonos Direct (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError</t>
+        </is>
+      </c>
+      <c r="W57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Sonos Direct</t>
+        </is>
+      </c>
+      <c r="Y57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="Z57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AB57" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>1 x single @ PayMore Murray ($141.99, snapshot, used) = $141.99 for 1 unit(s) ($141.99/unit); saves $68.01 vs 1 new singles</t>
+        </is>
+      </c>
+      <c r="AE57" s="11" t="n">
+        <v>141.99</v>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>GTIN 840136802846 | MPN/SKU RAYG1US1BLK | brand Sonos</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>verified_direct 1 | market_snapshot 4</t>
+        </is>
+      </c>
+      <c r="AH57" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>Yes (run 5 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>29</v>
+      </c>
+      <c r="F58" t="n">
+        <v>16</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>5</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" s="11" t="n">
+        <v>1104.13</v>
+      </c>
+      <c r="M58" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="O58" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 27 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
+        <v>7</v>
+      </c>
+      <c r="R58" t="n">
+        <v>7</v>
+      </c>
+      <c r="T58" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (cffi); identity validated (product_url)</t>
+        </is>
+      </c>
+      <c r="W58" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
+        </is>
+      </c>
+      <c r="Y58" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="Z58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AB58" s="11" t="n">
+        <v>1098.2</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>1 x single @ Google Shopping (several sellers) ($1,000.00, snapshot) = $1,000.00 for 1 unit(s) ($1,000.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE58" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>GTIN 887276934532 | MPN/SKU QN50QN90FAFXZA | brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 5</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | unavailable 1 (samsung.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>Yes (run 5 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Philips Hue Twilight Lamp Black</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="M59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="O59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (2 verified merchant prices; last discovery 6.0d ago (&lt; 6d) - credit saved) | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q59" t="n">
+        <v>2</v>
+      </c>
+      <c r="R59" t="n">
+        <v>2</v>
+      </c>
+      <c r="T59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Philips Hue Direct (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $319.99 stock unknown - visible price markup (cffi); identity validated (product_url) | philips-hue.com: [success] $319.99 in stock - JSON-LD; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
+        </is>
+      </c>
+      <c r="Y59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="Z59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA59" s="11" t="n">
+        <v>239.97</v>
+      </c>
+      <c r="AB59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>1 x single @ Philips Hue Direct ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE59" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>GTIN 46677585631 | MPN/SKU 929003711501 | brand Philips Hue</t>
+        </is>
+      </c>
+      <c r="AG59" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH59" t="inlineStr">
+        <is>
+          <t>success 2 | api_unavailable 1 (eBay) | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI59" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK59" t="inlineStr">
+        <is>
+          <t>Not run (SerpApi unavailable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>6</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" t="n">
+        <v>2</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="11" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="M60" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="O60" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (2 verified merchant prices; last discovery 6.0d ago (&lt; 6d) - credit saved)</t>
+        </is>
+      </c>
+      <c r="Q60" t="n">
+        <v>3</v>
+      </c>
+      <c r="R60" t="n">
+        <v>3</v>
+      </c>
+      <c r="T60" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Govee (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $169.99 stock unknown - visible price markup (browser render); identity validated (product_url) | us.govee.com: [success] $169.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
+        </is>
+      </c>
+      <c r="W60" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Govee</t>
+        </is>
+      </c>
+      <c r="Y60" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="Z60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA60" s="11" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="AB60" s="11" t="n">
+        <v>166.39</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>2 x single @ Govee ($169.99) = $339.98 for 2 unit(s) ($169.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE60" s="11" t="n">
+        <v>339.98</v>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>GTIN 810172723184 | MPN/SKU H1AA5, H1AA2 | brand Govee</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr">
+        <is>
+          <t>verified_direct 3</t>
+        </is>
+      </c>
+      <c r="AH60" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>11</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy Tab A9 plus silver</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>42</v>
+      </c>
+      <c r="F61" t="n">
+        <v>23</v>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="11" t="n">
+        <v>167.24</v>
+      </c>
+      <c r="O61" s="11" t="n">
+        <v>142.99</v>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Samsung, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | Avg (Resale) from only 2 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q61" t="n">
+        <v>11</v>
+      </c>
+      <c r="S61" t="n">
+        <v>2</v>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>ebay.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) | reebelo.com: [success] $153.28 in stock - JSON-LD; identity validated (product_url) (+2 variants)</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC61" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>1 x single @ eBay - scratchanddentdevices ($142.99, snapshot, used) = $142.99 for 1 unit(s) ($142.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE61" s="11" t="n">
+        <v>142.99</v>
+      </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG61" t="inlineStr">
+        <is>
+          <t>verified_direct 3 | market_snapshot 8</t>
+        </is>
+      </c>
+      <c r="AH61" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (ebay.com) | api_unavailable 1 (eBay) | skipped 5 (Dell, Home Depot, Microcenter, Samsung, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI61" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ61" t="inlineStr">
+        <is>
+          <t>Yes (run 4 in a row): ebay.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>12</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Geometric Plant Poster living room 28x40</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>40</v>
+      </c>
+      <c r="F62" t="n">
+        <v>17</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); no matching Etsy - Seller listing on Google Shopping | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) -&gt; no matching Etsy - Seller listing found via Google Shopping</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG62" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH62" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI62" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK62" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): Etsy - Seller (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>13</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>28x40” Walnut stain - Poster Frame</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | ArtToFrames.com: Product URL failed (identity_mismatch); ArtToFrames.com Google row used as market_snapshot | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q63" t="n">
+        <v>1</v>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>arttoframe.com: [identity_mismatch] $100.78 in stock - page is not this product - model '28x40' not in title; IDENTITY MISMATCH (excluded) -&gt; $88.53 from ArtToFrames.com via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG63" t="inlineStr">
+        <is>
+          <t>market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr">
+        <is>
+          <t>success 1 | identity_mismatch 1 (arttoframe.com) | timeout_network 1 (Google Shopping) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI63" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): arttoframe.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>14</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Teak Mid Century Modern Wall Pocket Set of 5</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>40</v>
+      </c>
+      <c r="F64" t="n">
+        <v>12</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); no matching Etsy - Seller listing on Google Shopping | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)) -&gt; no matching Etsy - Seller listing found via Google Shopping</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG64" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH64" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI64" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): Etsy - Seller (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>15</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>17 " H Faux Pampas Grass</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>38</v>
+      </c>
+      <c r="F65" t="n">
+        <v>26</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" s="11" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="O65" s="11" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Wayfair: Product URL failed (identity_mismatch); Wayfair Google row used as market_snapshot | SerpApi: success 40 listings | 4 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | Avg (New) from only 1 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q65" t="n">
+        <v>1</v>
+      </c>
+      <c r="R65" t="n">
+        <v>1</v>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>wayfair.com: [identity_mismatch] $39.99 stock unknown - page is not this product - Product URL page conflicts: different 17 model 'plant'; IDENTITY MISMATCH (excluded) -&gt; $45.99 from Wayfair via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>1 x single @ Wayfair ($45.99, snapshot) = $45.99 for 1 unit(s) ($45.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE65" s="11" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (wayfair.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): wayfair.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>16</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Farmhouse Full Length Mirror with Stand 22x65 Inch, Wooden Frame Floor Mirror</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Amazon: Product URL failed (identity_mismatch); same-vendor fallback no_match (live query) | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>amazon.com: [identity_mismatch] $129.59 stock unknown - page is not this product - model '22x65' not in title; IDENTITY MISMATCH (excluded) -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="W66" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y66" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="AA66" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="AB66" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
+          <t>no_match 1 (Amazon (Google Shopping)) | identity_mismatch 1 (amazon.com) | timeout_network 1 (Google Shopping) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>Yes: amazon.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK66" t="inlineStr">
+        <is>
+          <t>Yes: Amazon (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>17</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Vertical Bonsai Moss Wall Art</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>32</v>
+      </c>
+      <c r="F67" t="n">
+        <v>11</v>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="11" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="O67" s="11" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); Etsy - Seller Google row used as market_snapshot | SerpApi: success 40 listings | 9 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | Avg (New) from only 1 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q67" t="n">
+        <v>2</v>
+      </c>
+      <c r="R67" t="n">
+        <v>1</v>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)); browser: circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)) -&gt; $149.99 from Etsy - Seller via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>1 x single @ Etsy - Seller ($149.99, snapshot) = $149.99 for 1 unit(s) ($149.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE67" s="11" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t>market_snapshot 2</t>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI67" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ67" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>18</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>kasa ks225 light switch dimmers</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>41</v>
+      </c>
+      <c r="F68" t="n">
+        <v>23</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="O68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q68" t="n">
+        <v>1</v>
+      </c>
+      <c r="R68" t="n">
+        <v>1</v>
+      </c>
+      <c r="T68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $24.99 stock unknown - visible price markup (browser render); identity validated (mpn)</t>
+        </is>
+      </c>
+      <c r="W68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="Z68" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AB68" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>3 x single @ Amazon ($24.99) = $74.97 for 3 unit(s) ($24.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE68" s="11" t="n">
+        <v>74.97</v>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>MPN/SKU KS225 | brand Kasa</t>
+        </is>
+      </c>
+      <c r="AG68" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH68" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI68" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>19</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Motion Sensor</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" t="n">
+        <v>2</v>
+      </c>
+      <c r="I69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K69" s="11" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="O69" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (4 verified merchant prices; last discovery 6.0d ago (&lt; 6d) - credit saved)</t>
+        </is>
+      </c>
+      <c r="Q69" t="n">
+        <v>2</v>
+      </c>
+      <c r="R69" t="n">
+        <v>2</v>
+      </c>
+      <c r="T69" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $14.99 in stock - Shopify .js; identity validated (page_metadata) (+3 variants)</t>
+        </is>
+      </c>
+      <c r="W69" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y69" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="Z69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="AB69" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>5 x single @ THIRDREALITY Store ($14.99) = $74.95 for 5 unit(s) ($14.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE69" s="11" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1WMSA1 | brand ThirdReality</t>
+        </is>
+      </c>
+      <c r="AG69" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH69" t="inlineStr">
+        <is>
+          <t>success 1 | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI69" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK69" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>20</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Everything Presence One</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="n">
+        <v>2</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="O70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 1 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q70" t="n">
+        <v>1</v>
+      </c>
+      <c r="R70" t="n">
+        <v>1</v>
+      </c>
+      <c r="T70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>verified: everythingsmart.io (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>everythingsmart.io: [success] $64.00 in stock - Shopify .js; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at everythingsmart.io</t>
+        </is>
+      </c>
+      <c r="Y70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="Z70" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="AB70" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>2 x single @ everythingsmart.io ($64.00) = $128.00 for 2 unit(s) ($64.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE70" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>GTIN 5061109960010 | MPN/SKU EP1-FULL-01 | brand Everything Smart Technology</t>
+        </is>
+      </c>
+      <c r="AG70" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH70" t="inlineStr">
+        <is>
+          <t>success 2 | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>21</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Smart LV Wall Mount for Tablets</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>36</v>
+      </c>
+      <c r="F71" t="n">
+        <v>15</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | mount.modoco.io: Product URL failed (parser_failure); same-vendor fallback no_match (live query) | SerpApi: success 40 listings | 4 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>mount.modoco.io: [parser_failure] FAILED - no price data on page -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t>success 1 | no_match 1 (mount.modoco.io (Google Shopping)) | parser_failure 1 (mount.modoco.io) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): mount.modoco.io [parser_failure]</t>
+        </is>
+      </c>
+      <c r="AK71" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): mount.modoco.io (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>22</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Heat Wall Art</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>49</v>
+      </c>
+      <c r="F72" t="n">
+        <v>23</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="11" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | sandgrainstudio.com: Product URL failed (identity_mismatch); same-vendor fallback timeout_network (request failed) | SerpApi: success 40 listings | 3 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q72" t="n">
+        <v>6</v>
+      </c>
+      <c r="R72" t="n">
+        <v>4</v>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [identity_mismatch] $38.00 in stock - page is not this product - Product URL page conflicts: different heat model '30x45'; IDENTITY MISMATCH (excluded) (+11 variants) -&gt; same-vendor fallback: timeout_network (request failed)</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG72" t="inlineStr">
+        <is>
+          <t>market_snapshot 6</t>
+        </is>
+      </c>
+      <c r="AH72" t="inlineStr">
+        <is>
+          <t>success 1 | identity_mismatch 1 (heat) | timeout_network 1 (sandgrainstudio.com (Google Shopping)) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI72" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): sandgrainstudio.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>23</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>The Dark Knight Wall Art</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>49</v>
+      </c>
+      <c r="F73" t="n">
+        <v>12</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 40 listings | 3 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q73" t="n">
+        <v>16</v>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [success] $38.00 in stock - Shopify .js; identity unconfirmed - Medium, needs corroboration (not trusted) (+11 variants)</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG73" t="inlineStr">
+        <is>
+          <t>verified_direct 12 | market_snapshot 4</t>
+        </is>
+      </c>
+      <c r="AH73" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>24</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Dune Part 2 Wall Art</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>52</v>
+      </c>
+      <c r="F74" t="n">
+        <v>22</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q74" t="n">
+        <v>16</v>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [success] $38.00 in stock - Shopify .js; identity unconfirmed - Medium, needs corroboration (not trusted) (+11 variants)</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG74" t="inlineStr">
+        <is>
+          <t>verified_direct 12 | market_snapshot 4</t>
+        </is>
+      </c>
+      <c r="AH74" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n">
+        <v>46314.80508101852</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>25</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>12x18” Walnut stain - Poster Frame</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>41</v>
+      </c>
+      <c r="F75" t="n">
+        <v>19</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | arttoframe.com: Product URL failed (identity_mismatch); same-vendor fallback no_match (live query) | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q75" t="n">
+        <v>1</v>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>arttoframe.com: [identity_mismatch] $32.52 in stock - page is not this product - model '12x18' not in title; IDENTITY MISMATCH (excluded) -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC75" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t>market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH75" t="inlineStr">
+        <is>
+          <t>success 1 | no_match 1 (arttoframe.com (Google Shopping)) | identity_mismatch 1 (arttoframe.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): arttoframe.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK75" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): arttoframe.com (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -8561,7 +10816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF20"/>
+  <dimension ref="A1:AF29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -10376,7 +12631,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10416,8 +12670,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -10501,7 +12753,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -10538,8 +12789,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -10623,7 +12872,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -10663,8 +12911,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-13</t>
@@ -10748,7 +12994,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -10788,8 +13033,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-13</t>
@@ -10873,7 +13116,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -10913,8 +13155,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -10998,7 +13238,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11038,8 +13277,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -11053,6 +13290,1126 @@
       <c r="AF20" t="inlineStr">
         <is>
           <t>2026-10-16 17:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/smart-plug-gen3?variant=51228333867232</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>40.49</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>0.3253</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>below 30d verified median $13.49 [new pool]</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Smart Plug Gen3 - 4-Pack</t>
+        </is>
+      </c>
+      <c r="T21" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="U21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>verified_pack</t>
+        </is>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>7ae42c2156d2</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.google.com/shopping/product/11393094983587350623?gl=us&amp;hl=en</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>175</v>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Google Shopping (several sellers)</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="5" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>below 30d verified median $219.00; new verified low (prev $219.00) [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar (Black)</t>
+        </is>
+      </c>
+      <c r="T22" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U22" s="5" t="n">
+        <v>0.0411</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>title: exact name, no specs defined</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>85f07411c25b</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Sonos Ray Soundbar RAYG1US1BLK&amp;prds=catalogid:1268384348190922991,productid:3659965950609772637,headlineOfferDocid:15712000920323938156,imageDocid:15242818581710691365,rds:PC_29402159486281679|PROD_PC_29402159486281679,gpcid:29402159486281679,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>175</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>141.99</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PayMore Murray</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>used</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>141.99</v>
+      </c>
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="5" t="n">
+        <v>0.1886</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>&gt;=35% below new-condition regular/MSRP $219.00 [resale pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Google Shopping product rating 5.0/5 (104 reviews); product-level, not seller-level</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>SONOS Ray Compact Sound Bar</t>
+        </is>
+      </c>
+      <c r="T23" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U23" s="5" t="n">
+        <v>0.3516</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>title: exact name, no specs defined</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>6cf961b25227</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DXMVWFMC?plpRedirect=mhFallback&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
+        </is>
+      </c>
+      <c r="T24" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U24" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>64b642ed05e3</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.google.com/shopping/product/1015009314264515626?gl=us&amp;hl=en</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Google Shopping (several sellers)</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="5" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99; below 30d verified median $1097.99; new verified low (prev $1097.99) [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a WireLogic Ruby 8ft Ultra High Speed 4K-8K-10K HDMI Cable (2025)</t>
+        </is>
+      </c>
+      <c r="T25" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U25" s="5" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>83008cd05a0e</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:9212013035633147240,productid:507093706451136505,headlineOfferDocid:15716683707371333184,imageDocid:13820267211841367837,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G26" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L26" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
+        </is>
+      </c>
+      <c r="T26" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U26" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>21297db3f4f0</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:5203798915070718324,productid:16857903355191273450,headlineOfferDocid:13627928225093349671,imageDocid:10143191215087345269,gpcid:2544344569607442684,mid:576462914679857500,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
+      <c r="N27" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV Tilt-EXTENSION-37-90 Tilt Mount for 37"-90" TVs and Amber Protecti</t>
+        </is>
+      </c>
+      <c r="T27" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U27" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>e1df2775656a</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:3836802068298689922,productid:9032756040218221169,headlineOfferDocid:16228364667234284986,imageDocid:16792221860497270291,gpcid:8278254755523790402,mid:576462575320939649,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>1129.99</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="n">
+        <v>1129.99</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" s="5" t="n">
+        <v>-0.2555</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV Amber Protection Plan</t>
+        </is>
+      </c>
+      <c r="T28" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U28" s="5" t="n">
+        <v>0.2467</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>870e59980b4e</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>gh-39309907104</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>19</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Motion Sensor</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/motion-sensor?variant=48602222362848</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="5" t="n">
+        <v>0.2505</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $19.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Motion Sensor - Single Pack</t>
+        </is>
+      </c>
+      <c r="T29" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="U29" s="5" t="n">
+        <v>0.2501</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Y29" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-13</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>427b11691d77</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>2026-10-19 19:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price tracker: update run data (2026-10-22)
</commit_message>
<xml_diff>
--- a/Home Wishlist.xlsx
+++ b/Home Wishlist.xlsx
@@ -2131,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK75"/>
+  <dimension ref="A1:AK86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -10804,6 +10804,1313 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>17</v>
+      </c>
+      <c r="F76" t="n">
+        <v>13</v>
+      </c>
+      <c r="G76" t="n">
+        <v>2</v>
+      </c>
+      <c r="H76" t="n">
+        <v>2</v>
+      </c>
+      <c r="I76" t="n">
+        <v>1</v>
+      </c>
+      <c r="J76" t="n">
+        <v>1</v>
+      </c>
+      <c r="K76" s="11" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="M76" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="O76" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 15 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q76" t="n">
+        <v>3</v>
+      </c>
+      <c r="R76" t="n">
+        <v>3</v>
+      </c>
+      <c r="T76" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $13.49 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $40.49 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W76" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y76" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="Z76" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="AB76" s="11" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>2 x single @ THIRDREALITY Store ($13.49) = $26.98 for 2 unit(s) ($13.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE76" s="11" t="n">
+        <v>26.98</v>
+      </c>
+      <c r="AF76" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1SPD1Z, P1SPD4Z | brand THIRDREALITY</t>
+        </is>
+      </c>
+      <c r="AG76" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>success 3 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>14</v>
+      </c>
+      <c r="F77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="M77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="O77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 12 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q77" t="n">
+        <v>2</v>
+      </c>
+      <c r="R77" t="n">
+        <v>2</v>
+      </c>
+      <c r="T77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>verified: Sonos Direct (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $1,096.00 via Google Shopping fallback (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="W77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Sonos Direct</t>
+        </is>
+      </c>
+      <c r="Y77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="Z77" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AB77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>1 x single @ Sonos Direct ($219.00) = $219.00 for 1 unit(s) ($219.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE77" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AF77" t="inlineStr">
+        <is>
+          <t>GTIN 840136802846 | MPN/SKU RAYG1US1BLK | brand Sonos</t>
+        </is>
+      </c>
+      <c r="AG77" t="inlineStr">
+        <is>
+          <t>verified_direct 1 | market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH77" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI77" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>Yes (run 6 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>5</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>33</v>
+      </c>
+      <c r="F78" t="n">
+        <v>21</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" t="n">
+        <v>5</v>
+      </c>
+      <c r="J78" t="n">
+        <v>1</v>
+      </c>
+      <c r="K78" s="11" t="n">
+        <v>1116.16</v>
+      </c>
+      <c r="M78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="O78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 31 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q78" t="n">
+        <v>6</v>
+      </c>
+      <c r="R78" t="n">
+        <v>6</v>
+      </c>
+      <c r="T78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $2,000.00 via Google Shopping fallback (market_snapshot, not verified) | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (cffi); identity validated (product_url)</t>
+        </is>
+      </c>
+      <c r="W78" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
+        </is>
+      </c>
+      <c r="Y78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="Z78" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AB78" s="11" t="n">
+        <v>1098.13</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>1 x single @ Amazon ($1,097.99) = $1,097.99 for 1 unit(s) ($1,097.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE78" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AF78" t="inlineStr">
+        <is>
+          <t>GTIN 887276934532 | MPN/SKU QN50QN90FAFXZA | brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG78" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 4</t>
+        </is>
+      </c>
+      <c r="AH78" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | unavailable 1 (samsung.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI78" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ78" t="inlineStr">
+        <is>
+          <t>Yes (run 6 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>4</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Philips Hue Twilight Lamp Black</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>8</v>
+      </c>
+      <c r="F79" t="n">
+        <v>8</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="M79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="O79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 7 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Philips Hue Direct (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $319.99 stock unknown - visible price markup (browser render); identity validated (product_url) | philips-hue.com: [success] $319.99 in stock - JSON-LD; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
+        </is>
+      </c>
+      <c r="Y79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="Z79" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="11" t="n">
+        <v>239.97</v>
+      </c>
+      <c r="AB79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>1 x single @ Philips Hue Direct ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE79" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AF79" t="inlineStr">
+        <is>
+          <t>GTIN 46677585631 | MPN/SKU 929003711501 | brand Philips Hue</t>
+        </is>
+      </c>
+      <c r="AG79" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH79" t="inlineStr">
+        <is>
+          <t>success 3 | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI79" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>6</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>42</v>
+      </c>
+      <c r="F80" t="n">
+        <v>26</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2</v>
+      </c>
+      <c r="H80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="11" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="M80" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="O80" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q80" t="n">
+        <v>3</v>
+      </c>
+      <c r="R80" t="n">
+        <v>3</v>
+      </c>
+      <c r="T80" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Govee (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $169.99 stock unknown - visible price markup (browser render); identity validated (product_url) | us.govee.com: [success] $169.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
+        </is>
+      </c>
+      <c r="W80" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Govee</t>
+        </is>
+      </c>
+      <c r="Y80" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="Z80" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="11" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="AB80" s="11" t="n">
+        <v>167.47</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>2 x single @ Govee ($169.99) = $339.98 for 2 unit(s) ($169.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE80" s="11" t="n">
+        <v>339.98</v>
+      </c>
+      <c r="AF80" t="inlineStr">
+        <is>
+          <t>GTIN 810172723184 | MPN/SKU H1AA5, H1AA2 | brand Govee</t>
+        </is>
+      </c>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>verified_direct 3</t>
+        </is>
+      </c>
+      <c r="AH80" t="inlineStr">
+        <is>
+          <t>success 3 | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>11</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy Tab A9 plus silver</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>17</v>
+      </c>
+      <c r="F81" t="n">
+        <v>10</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>discovered[Samsung]: identity_mismatch - via sitemap: /us/mobile-accessories/galaxy-tab-s12-plus-pro-key: identity_mismatch; /us/tablets/galaxy-tab-s10-fe/buy/g | retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 11 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q81" t="n">
+        <v>7</v>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>ebay.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) | reebelo.com: [success] $140.99 in stock - JSON-LD; identity unconfirmed - Medium, needs corroboration (not trusted) (+5 variants)</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF81" t="inlineStr">
+        <is>
+          <t>brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>verified_direct 6 | market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (Samsung) | blocked 1 (ebay.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>Yes (run 5 in a row): ebay.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>8</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>6</v>
+      </c>
+      <c r="F82" t="n">
+        <v>6</v>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="n">
+        <v>1</v>
+      </c>
+      <c r="I82" t="n">
+        <v>1</v>
+      </c>
+      <c r="J82" t="n">
+        <v>1</v>
+      </c>
+      <c r="K82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="O82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | 6 Google row(s) from vendors with a working Product URL ignored | SerpApi: success 5 listings</t>
+        </is>
+      </c>
+      <c r="Q82" t="n">
+        <v>1</v>
+      </c>
+      <c r="R82" t="n">
+        <v>1</v>
+      </c>
+      <c r="T82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>verified: merachfit.com (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>merachfit.com: [success] $299.99 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W82" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>msrp_regular: retailer regular/list price at merachfit.com</t>
+        </is>
+      </c>
+      <c r="Y82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="Z82" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AB82" s="11" t="n">
+        <v>314.69</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>1 x single @ merachfit.com ($299.99) = $299.99 for 1 unit(s) ($299.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE82" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AF82" t="inlineStr">
+        <is>
+          <t>MPN/SKU MR-T25B2-US | brand MERACH</t>
+        </is>
+      </c>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH82" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI82" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>9</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Costway 47x24 Treadmill May Large</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | wayfair.com: Product URL failed (identity_mismatch); same-vendor fallback no_match (live query) | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q83" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>wayfair.com: [identity_mismatch] $29.99 stock unknown - page is not this product - Product URL page conflicts: accessory word 'protector'; IDENTITY MISMATCH (excluded) -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>brand Costway</t>
+        </is>
+      </c>
+      <c r="AG83" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH83" t="inlineStr">
+        <is>
+          <t>no_match 1 (wayfair.com (Google Shopping)) | identity_mismatch 1 (wayfair.com) | timeout_network 1 (Google Shopping) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>Yes (run 4 in a row): wayfair.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK83" t="inlineStr">
+        <is>
+          <t>Yes: wayfair.com (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>10</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Philips Hue Essential Smart LED A19 Bulb</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>41</v>
+      </c>
+      <c r="F84" t="n">
+        <v>26</v>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="n">
+        <v>1</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="O84" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>discovered[Philips Hue Direct]: identity_mismatch - via sitemap: /en-us/p/hue-white-and-color-ambiance-essential-a1: identity_mismatch; /en-us/p/bundle-bulb-ess | retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q84" t="n">
+        <v>1</v>
+      </c>
+      <c r="R84" t="n">
+        <v>1</v>
+      </c>
+      <c r="T84" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $17.50 stock unknown - visible price markup (browser render); identity validated (title)</t>
+        </is>
+      </c>
+      <c r="W84" s="11" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y84" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="Z84" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="AB84" s="11" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>2 x 4-pack @ Amazon ($17.50) = $35.00 for 8 unit(s) ($4.38/unit)</t>
+        </is>
+      </c>
+      <c r="AE84" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>MPN/SKU 592592 | brand Hue</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (Philips Hue Direct) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Kipp Glass Table Lamp - Walnut</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Article: Product URL failed (parser_failure); Article Google row used as market_snapshot | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q85" t="n">
+        <v>1</v>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>article.com: [parser_failure] FAILED - no price data on page -&gt; $149.00 from Article via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC85" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF85" t="inlineStr">
+        <is>
+          <t>MPN/SKU SKU27378 | brand Article</t>
+        </is>
+      </c>
+      <c r="AG85" t="inlineStr">
+        <is>
+          <t>market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH85" t="inlineStr">
+        <is>
+          <t>success 1 | timeout_network 1 (Google Shopping) | parser_failure 1 (article.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI85" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ85" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): article.com [parser_failure]</t>
+        </is>
+      </c>
+      <c r="AK85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n">
+        <v>46317.74858796296</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>7</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Japandi 3D Printed Reed Diffuser Container – Modern Organic Home Decor (Matte Finish)</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>21</v>
+      </c>
+      <c r="F86" t="n">
+        <v>4</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="11" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="O86" s="11" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); Etsy - Seller Google row used as market_snapshot | SerpApi: success 25 listings | 5 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | Avg (New) from only 1 listing(s): recorded, but deal rules need 3+</t>
+        </is>
+      </c>
+      <c r="Q86" t="n">
+        <v>1</v>
+      </c>
+      <c r="R86" t="n">
+        <v>1</v>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) -&gt; $17.99 from Etsy - Seller via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC86" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>3 x single @ Etsy - Seller ($17.99, snapshot) = $53.97 for 3 unit(s) ($17.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE86" s="11" t="n">
+        <v>53.97</v>
+      </c>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG86" t="inlineStr">
+        <is>
+          <t>market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH86" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI86" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ86" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -10816,7 +12123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF29"/>
+  <dimension ref="A1:AF36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -13360,7 +14667,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13400,8 +14706,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -13485,7 +14789,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -13522,8 +14825,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -13651,8 +14952,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
       <c r="AD23" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -13736,7 +15035,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -13773,8 +15071,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -13858,7 +15154,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -13895,8 +15190,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
       <c r="AD25" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -13980,7 +15273,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -14020,8 +15312,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
       <c r="AD26" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -14105,7 +15395,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -14145,8 +15434,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -14230,7 +15517,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -14270,8 +15556,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -14355,7 +15639,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -14395,8 +15678,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-13</t>
@@ -14410,6 +15691,878 @@
       <c r="AF29" t="inlineStr">
         <is>
           <t>2026-10-19 19:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/smart-plug-gen3?variant=51228333867232</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>40.49</v>
+      </c>
+      <c r="M30" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>0.3253</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>below 30d verified median $13.49 [new pool]</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Smart Plug Gen3 - 4-Pack</t>
+        </is>
+      </c>
+      <c r="T30" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="U30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>verified_pack</t>
+        </is>
+      </c>
+      <c r="Y30" s="11" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>7ae42c2156d2</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DXMVWFMC?plpRedirect=mhFallback&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G31" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
+        </is>
+      </c>
+      <c r="T31" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U31" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>64b642ed05e3</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:9212013035633147240,productid:507093706451136505,headlineOfferDocid:15716683707371333184,imageDocid:13820267211841367837,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M32" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
+        </is>
+      </c>
+      <c r="T32" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U32" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>21297db3f4f0</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:5203798915070718324,productid:16857903355191273450,headlineOfferDocid:13627928225093349671,imageDocid:10143191215087345269,gpcid:2544344569607442684,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L33" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV Tilt-EXTENSION-37-90 Tilt Mount for 37"-90" TVs and Amber Protecti</t>
+        </is>
+      </c>
+      <c r="T33" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U33" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z33" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-19</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>e1df2775656a</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=productid:15992245985528261990,headlineOfferDocid:15992245985528261990,imageDocid:6687171378154213687,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV FIXED-MOUNT-43-90 TV Mount for 43"-98" TVs and Amber Protection 3-</t>
+        </is>
+      </c>
+      <c r="T34" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U34" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z34" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>7e5ff0754d7d</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:15580681532640294837,productid:4764369165978523797,headlineOfferDocid:5018310726822602806,imageDocid:10130609959211192654,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" s="5" t="n">
+        <v>-0.3389</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Kanto R400 Recessed In-wall Full Motion Articulating Mount (2025)</t>
+        </is>
+      </c>
+      <c r="T35" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U35" s="5" t="n">
+        <v>0.1967</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-19</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>7418efe69185</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>gh-39827156585</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://merachfit.com/products/novawalk-w50-trekpad</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>merachfit.com</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+      <c r="N36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $479.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="T36" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="U36" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Y36" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>8fc2f05d8e66</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price tracker: update run data (2026-10-25)
</commit_message>
<xml_diff>
--- a/Home Wishlist.xlsx
+++ b/Home Wishlist.xlsx
@@ -2131,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK86"/>
+  <dimension ref="A1:AK106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12111,6 +12111,2249 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" t="n">
+        <v>2</v>
+      </c>
+      <c r="I87" t="n">
+        <v>1</v>
+      </c>
+      <c r="J87" t="n">
+        <v>1</v>
+      </c>
+      <c r="K87" s="11" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="M87" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="O87" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: timeout_network 0 listings (request failed) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q87" t="n">
+        <v>2</v>
+      </c>
+      <c r="R87" t="n">
+        <v>2</v>
+      </c>
+      <c r="T87" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $13.49 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $40.49 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W87" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y87" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="Z87" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="AB87" s="11" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>2 x single @ THIRDREALITY Store ($13.49) = $26.98 for 2 unit(s) ($13.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE87" s="11" t="n">
+        <v>26.98</v>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1SPD1Z, P1SPD4Z | brand THIRDREALITY</t>
+        </is>
+      </c>
+      <c r="AG87" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH87" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (Google Shopping) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI87" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>18</v>
+      </c>
+      <c r="F88" t="n">
+        <v>11</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" t="n">
+        <v>1</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" s="11" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="M88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="O88" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 16 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q88" t="n">
+        <v>2</v>
+      </c>
+      <c r="R88" t="n">
+        <v>2</v>
+      </c>
+      <c r="T88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>verified: Sonos Direct (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $1,096.00 via Google Shopping fallback (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="W88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Sonos Direct</t>
+        </is>
+      </c>
+      <c r="Y88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="Z88" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AB88" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>1 x single @ Google Shopping (several sellers) ($210.00, snapshot) = $210.00 for 1 unit(s) ($210.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE88" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>GTIN 840136802846 | MPN/SKU RAYG1US1BLK | brand Sonos</t>
+        </is>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>verified_direct 1 | market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH88" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI88" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ88" t="inlineStr">
+        <is>
+          <t>Yes (run 7 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>5</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>31</v>
+      </c>
+      <c r="F89" t="n">
+        <v>19</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="n">
+        <v>4</v>
+      </c>
+      <c r="J89" t="n">
+        <v>1</v>
+      </c>
+      <c r="K89" s="11" t="n">
+        <v>1119.79</v>
+      </c>
+      <c r="M89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="O89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 29 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q89" t="n">
+        <v>5</v>
+      </c>
+      <c r="R89" t="n">
+        <v>5</v>
+      </c>
+      <c r="T89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $2,000.00 via Google Shopping fallback (market_snapshot, not verified) | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (cffi); identity validated (product_url)</t>
+        </is>
+      </c>
+      <c r="W89" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
+        </is>
+      </c>
+      <c r="Y89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="Z89" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AB89" s="11" t="n">
+        <v>1098.09</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>1 x single @ Amazon ($1,097.99) = $1,097.99 for 1 unit(s) ($1,097.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE89" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
+          <t>GTIN 887276934532 | MPN/SKU QN50QN90FAFXZA | brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG89" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 3</t>
+        </is>
+      </c>
+      <c r="AH89" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | unavailable 1 (samsung.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ89" t="inlineStr">
+        <is>
+          <t>Yes (run 7 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>4</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Philips Hue Twilight Lamp Black</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="M90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="O90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (2 verified merchant prices; last discovery 3.0d ago (&lt; 6d) - credit saved) | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q90" t="n">
+        <v>2</v>
+      </c>
+      <c r="R90" t="n">
+        <v>2</v>
+      </c>
+      <c r="T90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Philips Hue Direct (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $319.99 stock unknown - visible price markup (cffi); identity validated (product_url) | philips-hue.com: [success] $319.99 in stock - JSON-LD; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
+        </is>
+      </c>
+      <c r="Y90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="Z90" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="11" t="n">
+        <v>239.97</v>
+      </c>
+      <c r="AB90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AC90" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>1 x single @ Philips Hue Direct ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE90" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>GTIN 46677585631 | MPN/SKU 929003711501 | brand Philips Hue</t>
+        </is>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH90" t="inlineStr">
+        <is>
+          <t>success 2 | api_unavailable 1 (eBay) | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>Not run (SerpApi unavailable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>6</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>35</v>
+      </c>
+      <c r="F91" t="n">
+        <v>23</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="n">
+        <v>1</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" s="11" t="n">
+        <v>134.99</v>
+      </c>
+      <c r="M91" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="O91" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 34 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q91" t="n">
+        <v>2</v>
+      </c>
+      <c r="R91" t="n">
+        <v>2</v>
+      </c>
+      <c r="T91" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>verified: Govee (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>amazon.com: [identity_mismatch] FAILED - stale link: redirected to a non-product page (https://www.amazon.com/checkpoint/continue?token=v1.6qm_3gHRk8CcZfuBDC1gagUFw2BLRhnpLXdf6I) | us.govee.com: [success] $169.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
+        </is>
+      </c>
+      <c r="W91" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Govee</t>
+        </is>
+      </c>
+      <c r="Y91" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="Z91" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA91" s="11" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="AB91" s="11" t="n">
+        <v>168.23</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>2 x single @ Govee ($169.99) = $339.98 for 2 unit(s) ($169.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE91" s="11" t="n">
+        <v>339.98</v>
+      </c>
+      <c r="AF91" t="inlineStr">
+        <is>
+          <t>GTIN 810172723184 | MPN/SKU H1AA5, H1AA2 | brand Govee</t>
+        </is>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (amazon.com) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ91" t="inlineStr">
+        <is>
+          <t>Yes: amazon.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>11</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy Tab A9 plus silver</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>12</v>
+      </c>
+      <c r="F92" t="n">
+        <v>7</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Samsung, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 7 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q92" t="n">
+        <v>6</v>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>ebay.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) | reebelo.com: [success] $153.28 in stock - JSON-LD; identity unconfirmed - Medium, needs corroboration (not trusted) (+4 variants)</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC92" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF92" t="inlineStr">
+        <is>
+          <t>brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG92" t="inlineStr">
+        <is>
+          <t>verified_direct 5 | market_snapshot 1</t>
+        </is>
+      </c>
+      <c r="AH92" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (ebay.com) | api_unavailable 1 (eBay) | skipped 5 (Dell, Home Depot, Microcenter, Samsung, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI92" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ92" t="inlineStr">
+        <is>
+          <t>Yes (run 6 in a row): ebay.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>12</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Geometric Plant Poster living room 28x40</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - LiberartAtelier: Product URL failed (blocked); no matching Etsy - LiberartAtelier listing on Google Shopping | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) -&gt; no matching Etsy - LiberartAtelier listing found via Google Shopping</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC93" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF93" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH93" t="inlineStr">
+        <is>
+          <t>success 1 | blocked 1 (etsy.com) | timeout_network 1 (Google Shopping) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI93" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ93" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK93" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): Etsy - LiberartAtelier (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>13</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>28x40” Walnut stain - Poster Frame</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>39</v>
+      </c>
+      <c r="F94" t="n">
+        <v>9</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | ArtToFrames.com: Product URL failed (identity_mismatch); ArtToFrames.com Google row used as market_snapshot | SerpApi: success 40 listings | 3 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q94" t="n">
+        <v>2</v>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>arttoframe.com: [identity_mismatch] $100.78 in stock - page is not this product - model '28x40' not in title; IDENTITY MISMATCH (excluded) -&gt; $88.53 from ArtToFrames.com via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC94" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF94" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>market_snapshot 2</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (arttoframe.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI94" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ94" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): arttoframe.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>14</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Teak Mid Century Modern Wall Pocket Set of 5</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>40</v>
+      </c>
+      <c r="F95" t="n">
+        <v>14</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); no matching Etsy - Seller listing on Google Shopping | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q95" t="n">
+        <v>0</v>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)) -&gt; no matching Etsy - Seller listing found via Google Shopping</t>
+        </is>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ95" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK95" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): Etsy - Seller (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>15</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>17 " H Faux Pampas Grass</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>42</v>
+      </c>
+      <c r="F96" t="n">
+        <v>12</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>2</v>
+      </c>
+      <c r="J96" t="n">
+        <v>2</v>
+      </c>
+      <c r="K96" s="11" t="n">
+        <v>63.74</v>
+      </c>
+      <c r="O96" s="11" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Wayfair: Product URL failed (identity_mismatch); Wayfair Google row used as market_snapshot | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q96" t="n">
+        <v>4</v>
+      </c>
+      <c r="R96" t="n">
+        <v>4</v>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>wayfair.com: [identity_mismatch] $39.99 stock unknown - page is not this product - Product URL page conflicts: different 17 model 'plant'; IDENTITY MISMATCH (excluded) -&gt; $21.99 from Wayfair via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="W96" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>regular_consensus: 2 listings publish a regular price</t>
+        </is>
+      </c>
+      <c r="AC96" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>1 x single @ Wayfair ($56.99, snapshot) = $56.99 for 1 unit(s) ($56.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE96" s="11" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>market_snapshot 4</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (wayfair.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): wayfair.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>16</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Farmhouse Full Length Mirror with Stand 22x65 Inch, Wooden Frame Floor Mirror</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>23</v>
+      </c>
+      <c r="F97" t="n">
+        <v>17</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="n">
+        <v>1</v>
+      </c>
+      <c r="I97" t="n">
+        <v>1</v>
+      </c>
+      <c r="J97" t="n">
+        <v>1</v>
+      </c>
+      <c r="K97" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="O97" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 22 listings | verified price down 15.0% vs prior $249.99 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="Q97" t="n">
+        <v>1</v>
+      </c>
+      <c r="R97" t="n">
+        <v>1</v>
+      </c>
+      <c r="T97" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $212.49 stock unknown - visible price markup (cffi); identity validated (title)</t>
+        </is>
+      </c>
+      <c r="W97" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y97" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="Z97" s="5" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="AA97" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="AB97" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>1 x single @ Amazon ($212.49) = $212.49 for 1 unit(s) ($212.49/unit)</t>
+        </is>
+      </c>
+      <c r="AE97" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI97" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>17</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Vertical Bonsai Moss Wall Art</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>36</v>
+      </c>
+      <c r="F98" t="n">
+        <v>8</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | Etsy - Seller: Product URL failed (blocked); Etsy - Seller Google row used as market_snapshot | SerpApi: success 40 listings | 5 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q98" t="n">
+        <v>0</v>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>etsy.com: [blocked] FAILED - circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)); browser: circuit open after 3 consecutive failures (site blocked automated access (HTTP 403)) -&gt; $73.50 from Etsy - Seller via Google Shopping (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC98" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (etsy.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI98" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ98" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): etsy.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>18</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>kasa ks225 light switch dimmers</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>38</v>
+      </c>
+      <c r="F99" t="n">
+        <v>19</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings | 2 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>amazon.com: [identity_mismatch] FAILED - stale link: redirected to a non-product page (https://www.amazon.com/checkpoint/continue?token=v1.hzJqnfeQzloaOiLdgOg2BTSsO0eMquTrlboBUL)</t>
+        </is>
+      </c>
+      <c r="W99" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>historical_verified: verified EWMA</t>
+        </is>
+      </c>
+      <c r="Y99" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AA99" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AB99" s="11" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>MPN/SKU KS225 | brand Kasa</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>success 1 | identity_mismatch 1 (amazon.com) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>Yes: amazon.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>19</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Motion Sensor</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>17</v>
+      </c>
+      <c r="F100" t="n">
+        <v>11</v>
+      </c>
+      <c r="G100" t="n">
+        <v>2</v>
+      </c>
+      <c r="H100" t="n">
+        <v>2</v>
+      </c>
+      <c r="I100" t="n">
+        <v>1</v>
+      </c>
+      <c r="J100" t="n">
+        <v>1</v>
+      </c>
+      <c r="K100" s="11" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="O100" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 13 listings</t>
+        </is>
+      </c>
+      <c r="Q100" t="n">
+        <v>4</v>
+      </c>
+      <c r="R100" t="n">
+        <v>4</v>
+      </c>
+      <c r="T100" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $14.99 in stock - Shopify .js; identity validated (page_metadata) (+3 variants)</t>
+        </is>
+      </c>
+      <c r="W100" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y100" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="Z100" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA100" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="AB100" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>5 x single @ THIRDREALITY Store ($14.99) = $74.95 for 5 unit(s) ($14.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE100" s="11" t="n">
+        <v>74.95</v>
+      </c>
+      <c r="AF100" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1WMSA1 | brand ThirdReality</t>
+        </is>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 2</t>
+        </is>
+      </c>
+      <c r="AH100" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI100" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>20</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Everything Presence One</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="O101" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 1 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q101" t="n">
+        <v>1</v>
+      </c>
+      <c r="R101" t="n">
+        <v>1</v>
+      </c>
+      <c r="T101" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>verified: everythingsmart.io (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>everythingsmart.io: [success] $65.00 in stock - Shopify .js; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W101" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at everythingsmart.io</t>
+        </is>
+      </c>
+      <c r="Y101" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="Z101" s="5" t="n">
+        <v>0.0156</v>
+      </c>
+      <c r="AA101" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="AB101" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>2 x single @ everythingsmart.io ($65.00) = $130.00 for 2 unit(s) ($65.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE101" s="11" t="n">
+        <v>130</v>
+      </c>
+      <c r="AF101" t="inlineStr">
+        <is>
+          <t>GTIN 5061109960010 | MPN/SKU EP1-FULL-01 | brand Everything Smart Technology</t>
+        </is>
+      </c>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH101" t="inlineStr">
+        <is>
+          <t>success 2 | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI101" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>21</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Smart LV Wall Mount for Tablets</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | mount.modoco.io: Product URL failed (parser_failure); same-vendor fallback no_match (live query) | SerpApi: timeout_network 0 listings (request failed)</t>
+        </is>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>mount.modoco.io: [parser_failure] FAILED - no price data on page -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC102" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF102" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG102" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>no_match 1 (mount.modoco.io (Google Shopping)) | timeout_network 1 (Google Shopping) | parser_failure 1 (mount.modoco.io) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI102" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ102" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): mount.modoco.io [parser_failure]</t>
+        </is>
+      </c>
+      <c r="AK102" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): mount.modoco.io (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>22</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Heat Wall Art</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>52</v>
+      </c>
+      <c r="F103" t="n">
+        <v>13</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" s="11" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | sandgrainstudio.com: Product URL failed (identity_mismatch); same-vendor fallback timeout_network (request failed) | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q103" t="n">
+        <v>6</v>
+      </c>
+      <c r="R103" t="n">
+        <v>6</v>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [identity_mismatch] $38.00 in stock - page is not this product - Product URL page conflicts: different heat model '30x45'; IDENTITY MISMATCH (excluded) (+11 variants) -&gt; same-vendor fallback: timeout_network (request failed)</t>
+        </is>
+      </c>
+      <c r="W103" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>regular_consensus: 4 listings publish a regular price</t>
+        </is>
+      </c>
+      <c r="AC103" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>market_snapshot 6</t>
+        </is>
+      </c>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>success 1 | identity_mismatch 1 (heat) | timeout_network 1 (sandgrainstudio.com (Google Shopping)) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI103" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ103" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): sandgrainstudio.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>23</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>The Dark Knight Wall Art</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>52</v>
+      </c>
+      <c r="F104" t="n">
+        <v>30</v>
+      </c>
+      <c r="G104" t="n">
+        <v>2</v>
+      </c>
+      <c r="H104" t="n">
+        <v>2</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" s="11" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="O104" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q104" t="n">
+        <v>28</v>
+      </c>
+      <c r="R104" t="n">
+        <v>8</v>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [success] $38.00 in stock - Shopify .js; identity unconfirmed - Medium, needs corroboration (not trusted) (+11 variants)</t>
+        </is>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC104" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>1 x single @ Best Buy ($19.99, snapshot) = $19.99 for 1 unit(s) ($19.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE104" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>verified_direct 12 | market_snapshot 16</t>
+        </is>
+      </c>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI104" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>24</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Dune Part 2 Wall Art</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>46</v>
+      </c>
+      <c r="F105" t="n">
+        <v>9</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | 6 Google row(s) from vendors with a working Product URL ignored | SerpApi: success 34 listings</t>
+        </is>
+      </c>
+      <c r="Q105" t="n">
+        <v>12</v>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>sandgrainstudio.com: [success] $38.00 in stock - Shopify .js; identity unconfirmed - Medium, needs corroboration (not trusted) (+11 variants)</t>
+        </is>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>verified_direct 12</t>
+        </is>
+      </c>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI105" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="n">
+        <v>46320.71049768518</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>25</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>12x18” Walnut stain - Poster Frame</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>35</v>
+      </c>
+      <c r="F106" t="n">
+        <v>19</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | ArtToFrames.com: Product URL failed (identity_mismatch); no matching ArtToFrames.com listing on Google Shopping | SerpApi: success 40 listings | 6 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>arttoframe.com: [identity_mismatch] $32.52 in stock - page is not this product - model '12x18' not in title; IDENTITY MISMATCH (excluded) -&gt; no matching ArtToFrames.com listing found via Google Shopping</t>
+        </is>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC106" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>title/spec matching only (no identifiers known yet)</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH106" t="inlineStr">
+        <is>
+          <t>success 2 | identity_mismatch 1 (arttoframe.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI106" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): arttoframe.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK106" t="inlineStr">
+        <is>
+          <t>Yes (run 3 in a row): ArtToFrames.com (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -12123,7 +14366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF36"/>
+  <dimension ref="A1:AF46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -15761,7 +18004,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -15801,8 +18043,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
       <c r="AD30" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -15886,7 +18126,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -15923,8 +18162,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
       <c r="AD31" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -16008,7 +18245,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -16048,8 +18284,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
       <c r="AD32" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -16133,7 +18367,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -16173,8 +18406,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-19</t>
@@ -16258,7 +18489,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -16298,8 +18528,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB34" t="inlineStr"/>
-      <c r="AC34" t="inlineStr"/>
       <c r="AD34" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -16383,7 +18611,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -16423,8 +18650,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
       <c r="AD35" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-19</t>
@@ -16508,7 +18733,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -16548,8 +18772,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -16563,6 +18785,1247 @@
       <c r="AF36" t="inlineStr">
         <is>
           <t>2026-10-22 17:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/smart-plug-gen3?variant=51228333867232</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G37" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>40.49</v>
+      </c>
+      <c r="M37" t="n">
+        <v>4</v>
+      </c>
+      <c r="N37" s="5" t="n">
+        <v>0.3253</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>below 30d verified median $13.49 [new pool]</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Smart Plug Gen3 - 4-Pack</t>
+        </is>
+      </c>
+      <c r="T37" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="U37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>verified_pack</t>
+        </is>
+      </c>
+      <c r="Y37" s="11" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>7ae42c2156d2</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.google.com/shopping/product/1388593028639213518?gl=us&amp;hl=en</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>175</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Google Shopping (several sellers)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L38" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
+      <c r="N38" s="5" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>below 30d verified median $219.00; new verified low (prev $219.00) [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Mastercard OFF | Sonos Ray Soundbar - Black</t>
+        </is>
+      </c>
+      <c r="T38" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U38" s="5" t="n">
+        <v>0.0411</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>title: exact name, no specs defined</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>price drop from $270.00</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>b7db16cba0a1</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DXMVWFMC?plpRedirect=mhFallback&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
+        </is>
+      </c>
+      <c r="T39" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U39" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>64b642ed05e3</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=productid:15992245985528261990,headlineOfferDocid:15992245985528261990,imageDocid:6687171378154213687,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G40" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L40" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M40" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV FIXED-MOUNT-43-90 TV Mount for 43"-98" TVs and Amber Protection 3-</t>
+        </is>
+      </c>
+      <c r="T40" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U40" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-22</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>7e5ff0754d7d</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:9212013035633147240,productid:507093706451136505,headlineOfferDocid:15716683707371333184,imageDocid:13820267211841367837,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G41" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L41" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M41" t="n">
+        <v>1</v>
+      </c>
+      <c r="N41" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
+        </is>
+      </c>
+      <c r="T41" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U41" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>21297db3f4f0</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:15580681532640294837,productid:4764369165978523797,headlineOfferDocid:5018310726822602806,imageDocid:10130609959211192654,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L42" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" s="5" t="n">
+        <v>-0.3389</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Kanto R400 Recessed In-wall Full Motion Articulating Mount (2025)</t>
+        </is>
+      </c>
+      <c r="T42" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U42" s="5" t="n">
+        <v>0.1967</v>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z42" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-19</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>7418efe69185</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>15</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>17 " H Faux Pampas Grass</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=17 " H Faux Pampas Grass&amp;prds=catalogid:13537295321086214348,productid:15861670781674970710,headlineOfferDocid:16631917063711727633,imageDocid:11930379475454550850,gpcid:500748725227803751,mid:576462916608404851,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="G43" s="11" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Wayfair</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1</v>
+      </c>
+      <c r="N43" s="5" t="n">
+        <v>-0.4248</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular-price consensus $80.00 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Atoll 17 " H Faux Pampas Grass Plant Primrue Flowers/Leaves</t>
+        </is>
+      </c>
+      <c r="T43" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="U43" s="5" t="n">
+        <v>0.2876</v>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>title: exact name, no specs defined</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>regular_consensus</t>
+        </is>
+      </c>
+      <c r="Z43" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>661c5542446f</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>15</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17 " H Faux Pampas Grass</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=17 " H Faux Pampas Grass&amp;prds=catalogid:7346776846355257774,productid:15607332985332939398,headlineOfferDocid:9268767640910713622,imageDocid:11502966817718223479,rds:PC_16834470426278337363|PROD_PC_16834470426278337363,gpcid:16834470426278337363,mid:576462719527143516,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="G44" s="11" t="n">
+        <v>57.99</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Wayfair</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L44" s="11" t="n">
+        <v>57.99</v>
+      </c>
+      <c r="M44" t="n">
+        <v>1</v>
+      </c>
+      <c r="N44" s="5" t="n">
+        <v>-0.4498</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular-price consensus $80.00 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>17 " H Faux Pampas Grass Plant Primrue</t>
+        </is>
+      </c>
+      <c r="T44" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="U44" s="5" t="n">
+        <v>0.2751</v>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>title: exact name, no specs defined</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>regular_consensus</t>
+        </is>
+      </c>
+      <c r="Z44" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>3b2c0dbe3da1</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>16</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Farmhouse Full Length Mirror with Stand 22x65 Inch, Wooden Frame Floor Mirror</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/WallBeyond-Mounted-Bedroom-Leaning-Hanging/dp/B0D1FWGGJD/ref=sr_1_1?s=home-garden&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="11" t="n">
+        <v>215</v>
+      </c>
+      <c r="G45" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="n">
+        <v>212.49</v>
+      </c>
+      <c r="M45" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="5" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>&gt;=15% below verified history $249.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Amazon.com: WallBeyond Farmhouse Full Length Mirror with Stand 22x65 Inch, Wooden Frame Floor Mirror,for Bedroom, Entryway, Living Room(Natural) : Home &amp; Kitchen</t>
+        </is>
+      </c>
+      <c r="T45" s="11" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="U45" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>title: Product URL validated (exact name, no specs defined)</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>historical_verified</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>price drop from $249.99</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>d7dac62e796e</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>gh-40214527797</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>19</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Motion Sensor</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/motion-sensor?variant=48602222362848</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G46" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L46" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="M46" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="5" t="n">
+        <v>0.2505</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $19.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Motion Sensor - Single Pack</t>
+        </is>
+      </c>
+      <c r="T46" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="U46" s="5" t="n">
+        <v>0.2501</v>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Y46" s="11" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-13</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>427b11691d77</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>2026-10-25 17:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price tracker: update run data (2026-10-28)
</commit_message>
<xml_diff>
--- a/Home Wishlist.xlsx
+++ b/Home Wishlist.xlsx
@@ -2131,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK106"/>
+  <dimension ref="A1:AK115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -14354,6 +14354,1110 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>20</v>
+      </c>
+      <c r="F107" t="n">
+        <v>15</v>
+      </c>
+      <c r="G107" t="n">
+        <v>2</v>
+      </c>
+      <c r="H107" t="n">
+        <v>2</v>
+      </c>
+      <c r="I107" t="n">
+        <v>1</v>
+      </c>
+      <c r="J107" t="n">
+        <v>1</v>
+      </c>
+      <c r="K107" s="11" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="M107" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="O107" s="11" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | SerpApi: success 18 listings | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly) | verified price up 11.1% vs prior $13.49 (2026-10-25)</t>
+        </is>
+      </c>
+      <c r="Q107" t="n">
+        <v>5</v>
+      </c>
+      <c r="R107" t="n">
+        <v>5</v>
+      </c>
+      <c r="T107" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>verified: THIRDREALITY Store (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>thirdreality.com: [success] $14.99 in stock - Shopify .js; identity validated (page_metadata) (+1 variants) | thirdreality.com: [success] $44.99 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W107" s="11" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="Y107" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="Z107" s="5" t="n">
+        <v>0.1112</v>
+      </c>
+      <c r="AA107" s="11" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="AB107" s="11" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="AC107" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>2 x single @ THIRDREALITY Store ($14.99) = $29.98 for 2 unit(s) ($14.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE107" s="11" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>MPN/SKU P1SPD1Z, P1SPD4Z | brand THIRDREALITY</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 3</t>
+        </is>
+      </c>
+      <c r="AH107" t="inlineStr">
+        <is>
+          <t>success 3 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI107" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>2</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Sonos Ray Soundbar</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>11</v>
+      </c>
+      <c r="F108" t="n">
+        <v>6</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="M108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="O108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 10 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q108" t="n">
+        <v>1</v>
+      </c>
+      <c r="R108" t="n">
+        <v>1</v>
+      </c>
+      <c r="T108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>verified: Sonos Direct (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>sonos.com: [success] $219.00 in stock - JSON-LD; identity validated (gtin) (+1 variants) | bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $1,096.00 via Google Shopping fallback (market_snapshot, not verified)</t>
+        </is>
+      </c>
+      <c r="W108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Sonos Direct</t>
+        </is>
+      </c>
+      <c r="Y108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="Z108" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AB108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AC108" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>1 x single @ Sonos Direct ($219.00) = $219.00 for 1 unit(s) ($219.00/unit)</t>
+        </is>
+      </c>
+      <c r="AE108" s="11" t="n">
+        <v>219</v>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>GTIN 840136802846 | MPN/SKU RAYG1US1BLK | brand Sonos</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH108" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>Yes (run 8 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>5</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>31</v>
+      </c>
+      <c r="F109" t="n">
+        <v>17</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="n">
+        <v>4</v>
+      </c>
+      <c r="J109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" s="11" t="n">
+        <v>1145.19</v>
+      </c>
+      <c r="M109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="O109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 29 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q109" t="n">
+        <v>5</v>
+      </c>
+      <c r="R109" t="n">
+        <v>5</v>
+      </c>
+      <c r="T109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>bestbuy.com: [timeout_network] FAILED - Chrome impersonation HTTPError -&gt; $2,000.00 via Google Shopping fallback (market_snapshot, not verified) | samsung.com: [unavailable] $1,099.99 OUT OF STOCK - JSON-LD; identity validated (brand_site) | amazon.com: [success] $1,097.99 stock unknown - visible price markup (browser render); identity validated (product_url)</t>
+        </is>
+      </c>
+      <c r="W109" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer regular/compare-at at Samsung</t>
+        </is>
+      </c>
+      <c r="Y109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="Z109" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AB109" s="11" t="n">
+        <v>1098.06</v>
+      </c>
+      <c r="AC109" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>1 x single @ Amazon ($1,097.99) = $1,097.99 for 1 unit(s) ($1,097.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE109" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="AF109" t="inlineStr">
+        <is>
+          <t>GTIN 887276934532 | MPN/SKU QN50QN90FAFXZA | brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG109" t="inlineStr">
+        <is>
+          <t>verified_direct 2 | market_snapshot 3</t>
+        </is>
+      </c>
+      <c r="AH109" t="inlineStr">
+        <is>
+          <t>success 2 | timeout_network 1 (bestbuy.com) | unavailable 1 (samsung.com) | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI109" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t>Yes (run 8 in a row): bestbuy.com [timeout_network]</t>
+        </is>
+      </c>
+      <c r="AK109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Philips Hue Twilight Lamp Black</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>6</v>
+      </c>
+      <c r="F110" t="n">
+        <v>5</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="M110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="O110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 5 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending)) | 1 duplicate row(s) merged as corroboration (same offer from another source, e.g. a Google row for a store already priced directly)</t>
+        </is>
+      </c>
+      <c r="Q110" t="n">
+        <v>2</v>
+      </c>
+      <c r="R110" t="n">
+        <v>2</v>
+      </c>
+      <c r="T110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Philips Hue Direct (page) (median of 2)</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $319.99 stock unknown - visible price markup (cffi); identity validated (product_url) | philips-hue.com: [success] $319.99 in stock - JSON-LD; identity validated (gtin)</t>
+        </is>
+      </c>
+      <c r="W110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Philips Hue Direct</t>
+        </is>
+      </c>
+      <c r="Y110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="Z110" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA110" s="11" t="n">
+        <v>239.97</v>
+      </c>
+      <c r="AB110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AC110" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>1 x single @ Philips Hue Direct ($319.99) = $319.99 for 1 unit(s) ($319.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE110" s="11" t="n">
+        <v>319.99</v>
+      </c>
+      <c r="AF110" t="inlineStr">
+        <is>
+          <t>GTIN 46677585631 | MPN/SKU 929003711501 | brand Philips Hue</t>
+        </is>
+      </c>
+      <c r="AG110" t="inlineStr">
+        <is>
+          <t>verified_direct 2</t>
+        </is>
+      </c>
+      <c r="AH110" t="inlineStr">
+        <is>
+          <t>success 3 | api_unavailable 1 (eBay) | skipped 4 (Dell, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI110" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>6</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>3</v>
+      </c>
+      <c r="F111" t="n">
+        <v>2</v>
+      </c>
+      <c r="G111" t="n">
+        <v>3</v>
+      </c>
+      <c r="H111" t="n">
+        <v>3</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3</v>
+      </c>
+      <c r="J111" t="n">
+        <v>3</v>
+      </c>
+      <c r="K111" s="11" t="n">
+        <v>124.32</v>
+      </c>
+      <c r="M111" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="O111" s="11" t="n">
+        <v>84.98999999999999</v>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: skipped 0 listings (3 verified merchant prices; last discovery 3.1d ago (&lt; 6d) - credit saved) | verified price down 15.3% vs prior $169.99 (2026-10-25)</t>
+        </is>
+      </c>
+      <c r="Q111" t="n">
+        <v>3</v>
+      </c>
+      <c r="R111" t="n">
+        <v>3</v>
+      </c>
+      <c r="T111" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page), Govee (page) (median of 3)</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $143.99 stock unknown - visible price markup (browser render); identity validated (product_url) | us.govee.com: [success] $143.99 in stock - JSON-LD; identity validated (brand_site) (+1 variants)</t>
+        </is>
+      </c>
+      <c r="W111" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>msrp_regular: manufacturer price at Govee</t>
+        </is>
+      </c>
+      <c r="Y111" s="11" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="Z111" s="5" t="n">
+        <v>-0.153</v>
+      </c>
+      <c r="AA111" s="11" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="AB111" s="11" t="n">
+        <v>168.75</v>
+      </c>
+      <c r="AC111" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>2 x single @ Govee ($84.99) = $169.98 for 2 unit(s) ($84.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE111" s="11" t="n">
+        <v>169.98</v>
+      </c>
+      <c r="AF111" t="inlineStr">
+        <is>
+          <t>GTIN 810172723184 | MPN/SKU H1AA5, H1AA2 | brand Govee</t>
+        </is>
+      </c>
+      <c r="AG111" t="inlineStr">
+        <is>
+          <t>verified_direct 3</t>
+        </is>
+      </c>
+      <c r="AH111" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 5 (Dell, Google Shopping, Home Depot, Microcenter, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI111" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK111" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>11</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy Tab A9 plus silver</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>17</v>
+      </c>
+      <c r="F112" t="n">
+        <v>12</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Samsung, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 13 listings | eBay: api_unavailable (EBAY_CLIENT_ID/EBAY_CLIENT_SECRET not set (optional - API access pending))</t>
+        </is>
+      </c>
+      <c r="Q112" t="n">
+        <v>6</v>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>ebay.com: [blocked] FAILED - site blocked automated access (HTTP 403); browser: site blocked automated access (HTTP 403) | reebelo.com: [success] $153.28 in stock - JSON-LD; identity unconfirmed - Medium, needs corroboration (not trusted) (+3 variants)</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC112" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF112" t="inlineStr">
+        <is>
+          <t>brand Samsung</t>
+        </is>
+      </c>
+      <c r="AG112" t="inlineStr">
+        <is>
+          <t>verified_direct 4 | market_snapshot 2</t>
+        </is>
+      </c>
+      <c r="AH112" t="inlineStr">
+        <is>
+          <t>success 2 | blocked 1 (ebay.com) | api_unavailable 1 (eBay) | skipped 5 (Dell, Home Depot, Microcenter, Samsung, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI112" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ112" t="inlineStr">
+        <is>
+          <t>Yes (run 7 in a row): ebay.com [blocked]</t>
+        </is>
+      </c>
+      <c r="AK112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F113" t="n">
+        <v>3</v>
+      </c>
+      <c r="G113" t="n">
+        <v>1</v>
+      </c>
+      <c r="H113" t="n">
+        <v>1</v>
+      </c>
+      <c r="I113" t="n">
+        <v>1</v>
+      </c>
+      <c r="J113" t="n">
+        <v>1</v>
+      </c>
+      <c r="K113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="O113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | 1 Google row(s) from vendors with a working Product URL ignored | SerpApi: success 3 listings</t>
+        </is>
+      </c>
+      <c r="Q113" t="n">
+        <v>1</v>
+      </c>
+      <c r="R113" t="n">
+        <v>1</v>
+      </c>
+      <c r="T113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>verified: merachfit.com (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>merachfit.com: [success] $299.99 in stock - Shopify .js; identity validated (page_metadata)</t>
+        </is>
+      </c>
+      <c r="W113" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>msrp_regular: retailer regular/list price at merachfit.com</t>
+        </is>
+      </c>
+      <c r="Y113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="Z113" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AB113" s="11" t="n">
+        <v>310.28</v>
+      </c>
+      <c r="AC113" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>1 x single @ merachfit.com ($299.99) = $299.99 for 1 unit(s) ($299.99/unit)</t>
+        </is>
+      </c>
+      <c r="AE113" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>MPN/SKU MR-T25B2-US | brand MERACH</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH113" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI113" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (1 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>9</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Costway 47x24 Treadmill May Large</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>41</v>
+      </c>
+      <c r="F114" t="n">
+        <v>13</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Only Check Primary Links = Yes: vendor lists, retailer discovery and eBay skipped | wayfair.com: Product URL failed (identity_mismatch); same-vendor fallback no_match (live query) | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>none (no verified merchant page/API priced the product)</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>wayfair.com: [identity_mismatch] $77.26 stock unknown - page is not this product - Product URL page conflicts: accessory word 'protector'; IDENTITY MISMATCH (excluded) -&gt; same-vendor fallback: no_match (live query)</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC114" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>no purchasable High-confidence offer</t>
+        </is>
+      </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>brand Costway</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr">
+        <is>
+          <t>no eligible listings</t>
+        </is>
+      </c>
+      <c r="AH114" t="inlineStr">
+        <is>
+          <t>success 1 | no_match 1 (wayfair.com (Google Shopping)) | identity_mismatch 1 (wayfair.com) | skipped 1 (vendor lists + retailer discovery + eBay)</t>
+        </is>
+      </c>
+      <c r="AI114" t="inlineStr">
+        <is>
+          <t>Product URLs + expanded SerpApi search (0 of 3 vendor links work)</t>
+        </is>
+      </c>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>Yes (run 5 in a row): wayfair.com [identity_mismatch]</t>
+        </is>
+      </c>
+      <c r="AK114" t="inlineStr">
+        <is>
+          <t>Yes (run 2 in a row): wayfair.com (same-vendor Google Shopping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="n">
+        <v>46323.78508101852</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>10</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Philips Hue Essential Smart LED A19 Bulb</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>41</v>
+      </c>
+      <c r="F115" t="n">
+        <v>19</v>
+      </c>
+      <c r="G115" t="n">
+        <v>1</v>
+      </c>
+      <c r="H115" t="n">
+        <v>1</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="M115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="O115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>retailer search skipped (never produced a listing): Philips Hue Direct, Home Depot, SuperBrightLEDs, Dell, Microcenter; Google Shopping still covers them | SerpApi: success 40 listings</t>
+        </is>
+      </c>
+      <c r="Q115" t="n">
+        <v>1</v>
+      </c>
+      <c r="R115" t="n">
+        <v>1</v>
+      </c>
+      <c r="T115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>verified: Amazon (page) (median of 1)</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>amazon.com: [success] $17.50 stock unknown - visible price markup (browser render); identity validated (title)</t>
+        </is>
+      </c>
+      <c r="W115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>historical_verified: 30-day verified median (3 runs)</t>
+        </is>
+      </c>
+      <c r="Y115" s="11" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="Z115" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="11" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="AB115" s="11" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="AC115" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD115" t="inlineStr">
+        <is>
+          <t>2 x 4-pack @ Amazon ($17.50) = $35.00 for 8 unit(s) ($4.38/unit)</t>
+        </is>
+      </c>
+      <c r="AE115" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="AF115" t="inlineStr">
+        <is>
+          <t>MPN/SKU 592592 | brand Hue</t>
+        </is>
+      </c>
+      <c r="AG115" t="inlineStr">
+        <is>
+          <t>verified_direct 1</t>
+        </is>
+      </c>
+      <c r="AH115" t="inlineStr">
+        <is>
+          <t>success 2 | skipped 5 (Dell, Home Depot, Microcenter, Philips Hue Direct, SuperBrightLEDs)</t>
+        </is>
+      </c>
+      <c r="AI115" t="inlineStr">
+        <is>
+          <t>Normal search</t>
+        </is>
+      </c>
+      <c r="AJ115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -14366,7 +15470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF46"/>
+  <dimension ref="A1:AF55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -18855,7 +19959,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -18895,8 +19998,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
       <c r="AD37" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-10</t>
@@ -18980,7 +20081,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19017,8 +20117,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="inlineStr">
         <is>
           <t>price drop from $270.00</t>
@@ -19102,7 +20200,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19139,8 +20236,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -19224,7 +20319,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19264,8 +20358,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-22</t>
@@ -19349,7 +20441,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19389,8 +20480,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB41" t="inlineStr"/>
-      <c r="AC41" t="inlineStr"/>
       <c r="AD41" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-03</t>
@@ -19474,7 +20563,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19514,8 +20602,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB42" t="inlineStr"/>
-      <c r="AC42" t="inlineStr"/>
       <c r="AD42" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-19</t>
@@ -19599,7 +20685,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19639,8 +20724,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB43" t="inlineStr"/>
-      <c r="AC43" t="inlineStr"/>
       <c r="AD43" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -19724,7 +20807,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19764,8 +20846,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB44" t="inlineStr"/>
-      <c r="AC44" t="inlineStr"/>
       <c r="AD44" t="inlineStr">
         <is>
           <t>new offer</t>
@@ -19849,7 +20929,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -19886,8 +20965,6 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="AB45" t="inlineStr"/>
-      <c r="AC45" t="inlineStr"/>
       <c r="AD45" t="inlineStr">
         <is>
           <t>price drop from $249.99</t>
@@ -19971,7 +21048,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -20011,8 +21087,6 @@
           <t>in_stock</t>
         </is>
       </c>
-      <c r="AB46" t="inlineStr"/>
-      <c r="AC46" t="inlineStr"/>
       <c r="AD46" t="inlineStr">
         <is>
           <t>unchanged since 2026-10-13</t>
@@ -20026,6 +21100,1116 @@
       <c r="AF46" t="inlineStr">
         <is>
           <t>2026-10-25 17:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Smart Plug Gen3</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.thirdreality.com/products/smart-plug-gen3?variant=51228333867232</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G47" s="11" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>THIRDREALITY Store</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L47" s="11" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="M47" t="n">
+        <v>4</v>
+      </c>
+      <c r="N47" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>below 30d verified median $13.49 [new pool]</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Smart Plug Gen3 - 4-Pack</t>
+        </is>
+      </c>
+      <c r="T47" s="11" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="U47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>verified_pack</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>price increase from $10.12</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>7ae42c2156d2</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DXMVWFMC?plpRedirect=mhFallback&amp;th=1</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G48" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L48" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M48" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Amazon.com: Samsung 50-Inch Class Neo QLED 4K QN90F Series, Vision AI, Mini LED Smart TV (2025 Model, 50QN90F) Neo Quantum HDR+, Object Tracking Sound Lite w/Dolby Atmos, Glare Free, Gaming Hub, Alexa</t>
+        </is>
+      </c>
+      <c r="T48" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U48" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>64b642ed05e3</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>5</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:9212013035633147240,productid:507093706451136505,headlineOfferDocid:15716683707371333184,imageDocid:13820267211841367837,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L49" s="11" t="n">
+        <v>1097.99</v>
+      </c>
+      <c r="M49" t="n">
+        <v>1</v>
+      </c>
+      <c r="N49" s="5" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Walts TV TILT-MOUNT-43-90 Large/XL Tilt Mount for 43"-98" TVs and Amber Pro</t>
+        </is>
+      </c>
+      <c r="T49" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U49" s="5" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z49" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-03</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>21297db3f4f0</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:15580681532640294837,productid:4764369165978523797,headlineOfferDocid:5018310726822602806,imageDocid:10130609959211192654,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G50" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L50" s="11" t="n">
+        <v>1204.99</v>
+      </c>
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" s="5" t="n">
+        <v>-0.3389</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with a Kanto R400 Recessed In-wall Full Motion Articulating Mount (2025)</t>
+        </is>
+      </c>
+      <c r="T50" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U50" s="5" t="n">
+        <v>0.1967</v>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z50" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-19</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>7418efe69185</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?ibp=oshop&amp;q=Samsung 50” QN90F Neo QLED Mini LED 4K UHD TV QN50QN90FAFXZA&amp;prds=catalogid:17601564680898175412,productid:9478909578281381128,headlineOfferDocid:12810016242466718140,imageDocid:9036445089217898831,pvt:hg&amp;hl=en&amp;gl=us&amp;udm=28</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G51" s="11" t="n">
+        <v>1224.99</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Newegg.com - Walts TV</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>serpapi</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L51" s="11" t="n">
+        <v>1224.99</v>
+      </c>
+      <c r="M51" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" s="5" t="n">
+        <v>-0.3611</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $1499.99 [new pool] [market snapshot - confirm on merchant page]</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Samsung QN50QN90FAFXZA 50 Inch Neo QLED 4K QN90F Vision AI Smart TV with an Austere 7S-8KHD2-2.5M VII Series 2.5m Premium Braided 8K HDMI Cable (2025)</t>
+        </is>
+      </c>
+      <c r="T51" s="11" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="U51" s="5" t="n">
+        <v>0.1833</v>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>market_snapshot</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>mpn: SKU/MPN + specs match</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Z51" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>new offer</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>da330bd88d5c</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://us.govee.com/products/govee-cob-strip-light-2-pro?variant=47771355742393</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="G52" s="11" t="n">
+        <v>84.98999999999999</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Govee</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="n">
+        <v>84.98999999999999</v>
+      </c>
+      <c r="M52" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="5" t="n">
+        <v>0.5001</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $143.99; below 30d verified median $169.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Govee COB Strip Light 2 Pro</t>
+        </is>
+      </c>
+      <c r="T52" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="U52" s="5" t="n">
+        <v>0.4098</v>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>brand_site: Product URL on the brand's own site (us.govee.com), no conflicts - Product URL identity unconfirmed (SKU/MPN match, some specs not in title)</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>price drop from $99.99; back in stock</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>bd2fbddb0fe4</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://us.govee.com/products/govee-cob-strip-light-2-pro?variant=47771355775161</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="G53" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Govee</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L53" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="M53" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" s="5" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>below 30d verified median $169.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Govee COB Strip Light 2 Pro</t>
+        </is>
+      </c>
+      <c r="T53" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="U53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>brand_site: Product URL on the brand's own site (us.govee.com), no conflicts - Product URL identity unconfirmed (SKU/MPN match, some specs not in title)</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>price drop from $169.99</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>f9e2ee8dc4ab</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Govee COB LED Strip Lights 2 Pro 16.4ft</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/Govee-Lights-RGBWWIC-1000K-10000K-16-4ft/dp/B0H6MBSRBT?th=1</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="G54" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L54" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="M54" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" s="5" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>below 30d verified median $169.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Amazon.com: Govee COB LED Strip Lights 2 Pro, RGBWWIC, 1344 LEDs/m, 1000K-10000K,16.4ft | Work with Alexa, Google Assistant, Matter and Smarthings, LuminBlend+, Cuttable, 540 lm/m, LED Lights for Bedr</t>
+        </is>
+      </c>
+      <c r="T54" s="11" t="n">
+        <v>143.99</v>
+      </c>
+      <c r="U54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>product_url: Product URL validated (title/slug match)</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>price drop from $169.99</t>
+        </is>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>75b7ca60a09a</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>gh-40748768157</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://merachfit.com/products/novawalk-w50-trekpad</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="G55" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>merachfit.com</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="L55" s="11" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M55" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>&gt;=15% below regular/MSRP $479.99 [new pool]</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>NovaWalk W50 TrekPad with 12% auto incline</t>
+        </is>
+      </c>
+      <c r="T55" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="U55" s="5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>verified_direct</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>page_metadata: Product URL validated (SKU/MPN + specs match)</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>msrp_regular</t>
+        </is>
+      </c>
+      <c r="Y55" s="11" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>unchanged since 2026-10-10</t>
+        </is>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>8fc2f05d8e66</t>
+        </is>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:51</t>
         </is>
       </c>
     </row>

</xml_diff>